<commit_message>
Add in-progress economics workstream files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K2weV5RtvDCshBNnABKa1E
</commit_message>
<xml_diff>
--- a/priyanka_nanda_academy/economics/market_sizing_model.xlsx
+++ b/priyanka_nanda_academy/economics/market_sizing_model.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="579">
   <si>
     <t xml:space="preserve">PNA market sizing model - TAM / SAM / SOM with tricity-India reconciliation</t>
   </si>
@@ -807,6 +807,24 @@
     <t xml:space="preserve">Y3 adjacent revenue outside the training market (kit margin, services desk, partnerships)</t>
   </si>
   <si>
+    <t xml:space="preserve">SOM-LRN-TRI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y3 tricity-origin career learners (L2+L3 new students)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOM-LRN-REG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y3 out-of-town career learners (offline + satellite)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOM-LRN-HYB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y3 incremental destination/hybrid learners</t>
+  </si>
+  <si>
     <t xml:space="preserve">SOM-BASELINE</t>
   </si>
   <si>
@@ -945,6 +963,9 @@
     <t xml:space="preserve">TAM: makeup-led paid tuition, India (₹ crore/yr)</t>
   </si>
   <si>
+    <t xml:space="preserve">equals CA-06 (₹80 / 390 / 1,370 crore)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Makeup-led paid learners, India (mean of methods)</t>
   </si>
   <si>
@@ -1104,6 +1125,9 @@
     <t xml:space="preserve">tricity counts students who come from home states</t>
   </si>
   <si>
+    <t xml:space="preserve">Tricity share of India makeup-led learners (product)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Method A learners</t>
   </si>
   <si>
@@ -1182,10 +1206,10 @@
     <t xml:space="preserve">  of which outstation (inflow) learners</t>
   </si>
   <si>
-    <t xml:space="preserve">Reconciled tricity share of India TAM (same case)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base ≈0.8-0.9% vs 1.5% apparent</t>
+    <t xml:space="preserve">Reconciled tricity revenue as share of India BASE TAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base ≈0.84% vs 1.46% apparent (CA-05/CA-06)</t>
   </si>
   <si>
     <t xml:space="preserve">Outer bounds: min of method lows / max of method highs (learners)</t>
@@ -1269,6 +1293,9 @@
     <t xml:space="preserve">Σ women (000)</t>
   </si>
   <si>
+    <t xml:space="preserve">equals X-W-ROR 12,376</t>
+  </si>
+  <si>
     <t xml:space="preserve">KPMG intensity index, rest of region</t>
   </si>
   <si>
@@ -1455,6 +1482,27 @@
     <t xml:space="preserve">Online (SAM-5): implied share of SAM component</t>
   </si>
   <si>
+    <t xml:space="preserve">Learner-share test (primary: PNA charges ~1.8x the tricity average fee, so revenue share overstates position)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNA Y3 tricity career learners / tricity makeup-led learners (SAM-1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chandigarh agent: 10-30% is the plausible single-centre band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNA Y3 out-of-town career learners / net regional reachable learners (SAM-2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">denominator incl. inflow already in tricity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNA Y3 hybrid learners / hybrid-willing learners (SAM-3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNA Y3 tricity career learners / CA-05 tricity learners (BM test: flag if &gt;10% without regional engine)</t>
+  </si>
+  <si>
     <t xml:space="preserve">SOM training total (₹ crore, quoted)</t>
   </si>
   <si>
@@ -1572,6 +1620,12 @@
     <t xml:space="preserve">  SOM as % of SAM core (excl. online)</t>
   </si>
   <si>
+    <t xml:space="preserve">  PNA learner share of tricity makeup-led learners (Y3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">primary share test</t>
+  </si>
+  <si>
     <t xml:space="preserve">  SOM as % of TAM incl. online</t>
   </si>
   <si>
@@ -1704,7 +1758,7 @@
     <t xml:space="preserve">SOM &lt; SAM total (all cases)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base SOM share of tricity &lt;= 25%</t>
+    <t xml:space="preserve">Base SOM learner share of tricity &lt;= 25% (revenue share shown separately)</t>
   </si>
   <si>
     <t xml:space="preserve">KPMG tricity intensity within 10% of affluence weight (cross-check)</t>
@@ -2393,7 +2447,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M84"/>
+  <dimension ref="A1:M87"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -4498,13 +4552,13 @@
         <v>245</v>
       </c>
       <c r="C78" s="16" t="n">
-        <v>0</v>
+        <v>19.51</v>
       </c>
       <c r="D78" s="16" t="n">
-        <v>0</v>
+        <v>71.87</v>
       </c>
       <c r="E78" s="16" t="n">
-        <v>0</v>
+        <v>104.57</v>
       </c>
       <c r="F78" s="10" t="s">
         <v>246</v>
@@ -4517,7 +4571,7 @@
       </c>
       <c r="I78" s="17" t="n">
         <f aca="false">INDEX(C78:E78,$C$4)</f>
-        <v>0</v>
+        <v>71.87</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4528,13 +4582,13 @@
         <v>250</v>
       </c>
       <c r="C79" s="16" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="D79" s="16" t="n">
-        <v>0</v>
+        <v>24.86</v>
       </c>
       <c r="E79" s="16" t="n">
-        <v>0</v>
+        <v>75.56</v>
       </c>
       <c r="F79" s="10" t="s">
         <v>246</v>
@@ -4547,7 +4601,7 @@
       </c>
       <c r="I79" s="17" t="n">
         <f aca="false">INDEX(C79:E79,$C$4)</f>
-        <v>0</v>
+        <v>24.86</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4558,13 +4612,13 @@
         <v>252</v>
       </c>
       <c r="C80" s="16" t="n">
-        <v>0</v>
+        <v>4.63</v>
       </c>
       <c r="D80" s="16" t="n">
-        <v>0</v>
+        <v>25.15</v>
       </c>
       <c r="E80" s="16" t="n">
-        <v>0</v>
+        <v>49.35</v>
       </c>
       <c r="F80" s="10" t="s">
         <v>246</v>
@@ -4577,7 +4631,7 @@
       </c>
       <c r="I80" s="17" t="n">
         <f aca="false">INDEX(C80:E80,$C$4)</f>
-        <v>0</v>
+        <v>25.15</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4588,13 +4642,13 @@
         <v>254</v>
       </c>
       <c r="C81" s="16" t="n">
-        <v>0</v>
+        <v>5.84</v>
       </c>
       <c r="D81" s="16" t="n">
-        <v>0</v>
+        <v>27.06</v>
       </c>
       <c r="E81" s="16" t="n">
-        <v>0</v>
+        <v>61.15</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>246</v>
@@ -4607,7 +4661,7 @@
       </c>
       <c r="I81" s="17" t="n">
         <f aca="false">INDEX(C81:E81,$C$4)</f>
-        <v>0</v>
+        <v>27.06</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4618,13 +4672,13 @@
         <v>256</v>
       </c>
       <c r="C82" s="16" t="n">
-        <v>0</v>
+        <v>1.27</v>
       </c>
       <c r="D82" s="16" t="n">
-        <v>0</v>
+        <v>11.43</v>
       </c>
       <c r="E82" s="16" t="n">
-        <v>0</v>
+        <v>33.88</v>
       </c>
       <c r="F82" s="10" t="s">
         <v>246</v>
@@ -4637,7 +4691,7 @@
       </c>
       <c r="I82" s="17" t="n">
         <f aca="false">INDEX(C82:E82,$C$4)</f>
-        <v>0</v>
+        <v>11.43</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4648,13 +4702,13 @@
         <v>258</v>
       </c>
       <c r="C83" s="16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D83" s="16" t="n">
-        <v>0</v>
+        <v>6.55</v>
       </c>
       <c r="E83" s="16" t="n">
-        <v>0</v>
+        <v>10.13</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>246</v>
@@ -4667,37 +4721,127 @@
       </c>
       <c r="I83" s="17" t="n">
         <f aca="false">INDEX(C83:E83,$C$4)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>6.55</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
         <v>259</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>260</v>
       </c>
-      <c r="C84" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D84" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E84" s="16" t="n">
-        <v>0</v>
+      <c r="C84" s="9" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="D84" s="9" t="n">
+        <v>93.9</v>
+      </c>
+      <c r="E84" s="9" t="n">
+        <v>97.5</v>
       </c>
       <c r="F84" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H84" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="I84" s="11" t="n">
+        <f aca="false">INDEX(C84:E84,$C$4)</f>
+        <v>93.9</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="C85" s="9" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="D85" s="9" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="E85" s="9" t="n">
+        <v>95</v>
+      </c>
+      <c r="F85" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H85" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="I85" s="11" t="n">
+        <f aca="false">INDEX(C85:E85,$C$4)</f>
+        <v>40.2</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="C86" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="D86" s="9" t="n">
+        <v>35</v>
+      </c>
+      <c r="E86" s="9" t="n">
+        <v>53.9</v>
+      </c>
+      <c r="F86" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G86" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="H86" s="10" t="s">
+        <v>248</v>
+      </c>
+      <c r="I86" s="11" t="n">
+        <f aca="false">INDEX(C86:E86,$C$4)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="C87" s="16" t="n">
+        <v>6.71</v>
+      </c>
+      <c r="D87" s="16" t="n">
+        <v>16.61</v>
+      </c>
+      <c r="E87" s="16" t="n">
+        <v>24.92</v>
+      </c>
+      <c r="F87" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="G84" s="4" t="s">
-        <v>261</v>
-      </c>
-      <c r="H84" s="10" t="s">
+      <c r="G87" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="H87" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="I84" s="17" t="n">
-        <f aca="false">INDEX(C84:E84,$C$4)</f>
-        <v>0</v>
+      <c r="I87" s="17" t="n">
+        <f aca="false">INDEX(C87:E87,$C$4)</f>
+        <v>16.61</v>
       </c>
     </row>
   </sheetData>
@@ -4733,20 +4877,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -4758,12 +4902,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4773,10 +4917,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">Assumptions!$C$9</f>
@@ -4796,7 +4940,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">C6/Assumptions!$C$10</f>
@@ -4811,12 +4955,12 @@
         <v>525000</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">C7/Assumptions!$C$29</f>
@@ -4831,12 +4975,12 @@
         <v>0.772485962826504</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">Assumptions!$C$11</f>
@@ -4856,7 +5000,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">C7*C9</f>
@@ -4871,12 +5015,12 @@
         <v>420000</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="C11" s="25" t="n">
         <f aca="false">Assumptions!$C$12</f>
@@ -4896,7 +5040,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C12" s="26" t="n">
         <f aca="false">C10*C11</f>
@@ -4911,12 +5055,12 @@
         <v>147000</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="C13" s="27" t="n">
         <f aca="false">Assumptions!$C$13*Assumptions!$C$14+Assumptions!$C$15*Assumptions!$C$16+Assumptions!$C$17*Assumptions!$C$18+Assumptions!$C$19*Assumptions!$C$20</f>
@@ -4931,12 +5075,12 @@
         <v>109000</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="C14" s="28" t="n">
         <f aca="false">C12*C13/10000000</f>
@@ -4951,12 +5095,12 @@
         <v>1602.3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">C10-C12</f>
@@ -4971,12 +5115,12 @@
         <v>273000</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="C16" s="29" t="n">
         <f aca="false">C15*Assumptions!$C$21/10000000</f>
@@ -4991,12 +5135,12 @@
         <v>491.4</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="C17" s="29" t="n">
         <f aca="false">C14+C16</f>
@@ -5011,12 +5155,12 @@
         <v>2093.7</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -5026,7 +5170,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">Assumptions!$C$22</f>
@@ -5046,7 +5190,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="C21" s="24" t="n">
         <f aca="false">Assumptions!$C$23</f>
@@ -5066,7 +5210,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">C20*C21</f>
@@ -5081,12 +5225,12 @@
         <v>75000</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="C23" s="24" t="n">
         <f aca="false">C22*(1+Assumptions!$C$24)</f>
@@ -5101,12 +5245,12 @@
         <v>300000</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="C24" s="26" t="n">
         <f aca="false">C23*Assumptions!$C$12</f>
@@ -5121,12 +5265,12 @@
         <v>105000</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C25" s="28" t="n">
         <f aca="false">C24*C13/10000000</f>
@@ -5141,12 +5285,12 @@
         <v>1144.5</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">(C23-C24)*Assumptions!$C$21/10000000</f>
@@ -5164,7 +5308,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">C25+C26</f>
@@ -5182,7 +5326,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -5192,7 +5336,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="C30" s="28" t="n">
         <f aca="false">AVERAGE(C14,C25)</f>
@@ -5206,14 +5350,13 @@
         <f aca="false">AVERAGE(E14,E25)</f>
         <v>1373.4</v>
       </c>
-      <c r="F30" s="2" t="e">
-        <f aca="false">ca-6 (₹80 / 390 / 1,370 crore))</f>
-        <v>#N/A</v>
+      <c r="F30" s="2" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="C31" s="26" t="n">
         <f aca="false">AVERAGE(C12,C24)</f>
@@ -5228,12 +5371,12 @@
         <v>126000</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">C31/Assumptions!$C$33</f>
@@ -5248,12 +5391,12 @@
         <v>0.565164346203531</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C33" s="29" t="n">
         <f aca="false">Assumptions!$C$25*Assumptions!$C$26/10000000</f>
@@ -5268,12 +5411,12 @@
         <v>120</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C34" s="28" t="n">
         <f aca="false">C30+C33</f>
@@ -5291,7 +5434,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="C35" s="29" t="n">
         <f aca="false">C30*10000000/Assumptions!$C$27/1000000</f>
@@ -5306,12 +5449,12 @@
         <v>156.068181818182</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="C36" s="29" t="n">
         <f aca="false">AVERAGE(C17,C27)</f>
@@ -5326,12 +5469,12 @@
         <v>1794.6</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C37" s="25" t="n">
         <f aca="false">C30/Assumptions!$C$30</f>
@@ -5346,12 +5489,12 @@
         <v>0.0180375881588106</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">C30*Assumptions!$C$28</f>
@@ -5366,12 +5509,12 @@
         <v>105.0651</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
   </sheetData>
@@ -5401,20 +5544,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -5426,12 +5569,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5441,7 +5584,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="22" t="n">
@@ -5457,12 +5600,12 @@
         <v>2.55601659751037</v>
       </c>
       <c r="F6" s="30" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="22" t="n">
@@ -5481,7 +5624,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="22" t="n">
@@ -5500,7 +5643,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="24" t="n">
@@ -5516,12 +5659,12 @@
         <v>471</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="22" t="n">
@@ -5537,12 +5680,12 @@
         <v>2</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="10" t="n">
@@ -5561,7 +5704,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="31" t="n">
@@ -5577,12 +5720,12 @@
         <v>1.90293451735955</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5592,7 +5735,7 @@
     </row>
     <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="24" t="n">
@@ -5608,12 +5751,12 @@
         <v>2228.57142857143</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="31" t="n">
@@ -5629,12 +5772,12 @@
         <v>13.3714285714286</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="29" t="n">
@@ -5650,12 +5793,12 @@
         <v>1373.4</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="32" t="n">
@@ -5671,12 +5814,12 @@
         <v>0.00973600449354054</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="33" t="n">
@@ -5692,12 +5835,12 @@
         <v>0.00233242428591933</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -5707,7 +5850,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="24" t="n">
@@ -5723,12 +5866,12 @@
         <v>126000</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="33" t="n">
@@ -5747,7 +5890,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="22" t="n">
@@ -5763,12 +5906,12 @@
         <v>2.28</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="22" t="n">
@@ -5784,12 +5927,12 @@
         <v>1.83188405797101</v>
       </c>
       <c r="F25" s="30" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="22" t="n">
@@ -5805,13 +5948,12 @@
         <v>1.42857142857143</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="e">
-        <f aca="false">tricity share of india makeup-led learners</f>
-        <v>#VALUE!</v>
+      <c r="A27" s="3" t="s">
+        <v>365</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="32" t="n">
@@ -5830,7 +5972,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="26" t="n">
@@ -5849,7 +5991,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="22" t="n">
@@ -5865,12 +6007,12 @@
         <v>10.5211724839461</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -5880,7 +6022,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="24" t="n">
@@ -5899,7 +6041,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="25" t="n">
@@ -5915,12 +6057,12 @@
         <v>0.8</v>
       </c>
       <c r="F33" s="30" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="26" t="n">
@@ -5939,7 +6081,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="22" t="n">
@@ -5958,7 +6100,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -5968,7 +6110,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="24" t="n">
@@ -5984,12 +6126,12 @@
         <v>420</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="24" t="n">
@@ -6005,12 +6147,12 @@
         <v>300</v>
       </c>
       <c r="F39" s="30" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="23" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="24" t="n">
@@ -6026,12 +6168,12 @@
         <v>320</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="24" t="n">
@@ -6047,12 +6189,12 @@
         <v>133.2</v>
       </c>
       <c r="F41" s="30" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="26" t="n">
@@ -6071,7 +6213,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="22" t="n">
@@ -6090,7 +6232,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -6100,7 +6242,7 @@
     </row>
     <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="26" t="n">
@@ -6116,12 +6258,12 @@
         <v>879.2</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="31" t="n">
@@ -6137,12 +6279,12 @@
         <v>5.2752</v>
       </c>
       <c r="F47" s="30" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="24" t="n">
@@ -6161,28 +6303,28 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="32" t="n">
-        <f aca="false">C47/C17</f>
-        <v>0.0181828335400167</v>
+        <f aca="false">C47/$D$17</f>
+        <v>0.00374669375987229</v>
       </c>
       <c r="D49" s="32" t="n">
-        <f aca="false">D47/D17</f>
+        <f aca="false">D47/$D$17</f>
         <v>0.0084270044434947</v>
       </c>
       <c r="E49" s="32" t="n">
-        <f aca="false">E47/E17</f>
-        <v>0.00384097859327217</v>
+        <f aca="false">E47/$D$17</f>
+        <v>0.0136048066345096</v>
       </c>
       <c r="F49" s="30" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="23" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="24" t="n">
@@ -6198,12 +6340,12 @@
         <v>1782.85714285714</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -6213,7 +6355,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="22" t="n">
@@ -6232,7 +6374,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="23" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="22" t="n">
@@ -6251,7 +6393,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="34" t="n">
@@ -6270,7 +6412,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="35" t="n">
@@ -6289,7 +6431,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="35" t="n">
@@ -6308,7 +6450,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="23" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="35" t="n">
@@ -6327,7 +6469,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="23" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="35" t="n">
@@ -6346,7 +6488,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="34" t="n">
@@ -6365,7 +6507,7 @@
     </row>
     <row r="61" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="34" t="n">
@@ -6381,12 +6523,12 @@
         <v>1.01672535769804</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="23" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="35" t="n">
@@ -6402,12 +6544,12 @@
         <v>1.49945613983708</v>
       </c>
       <c r="F62" s="30" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -6417,7 +6559,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="36" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="B65" s="36"/>
       <c r="C65" s="36"/>
@@ -6427,7 +6569,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="36" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="B66" s="36"/>
       <c r="C66" s="36"/>
@@ -6437,7 +6579,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="36" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="B67" s="36"/>
       <c r="C67" s="36"/>
@@ -6447,7 +6589,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="36" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="B68" s="36"/>
       <c r="C68" s="36"/>
@@ -6457,7 +6599,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="36" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="B69" s="36"/>
       <c r="C69" s="36"/>
@@ -6467,7 +6609,7 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="36" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="B70" s="36"/>
       <c r="C70" s="36"/>
@@ -6510,20 +6652,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -6535,12 +6677,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -6550,7 +6692,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">(Assumptions!$C$38*Assumptions!$C$44+Assumptions!$C$39*Assumptions!$C$45+Assumptions!$C$40*Assumptions!$C$46+Assumptions!$C$41*Assumptions!$C$47)/Assumptions!$C$42</f>
@@ -6568,7 +6710,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">Assumptions!$C$38+Assumptions!$C$39+Assumptions!$C$40+Assumptions!$C$41</f>
@@ -6582,14 +6724,13 @@
         <f aca="false">Assumptions!$E$38+Assumptions!$E$39+Assumptions!$E$40+Assumptions!$E$41</f>
         <v>12376</v>
       </c>
-      <c r="F7" s="2" t="e">
-        <f aca="false">x-w-ror 12,376</f>
-        <v>#VALUE!</v>
+      <c r="F7" s="2" t="s">
+        <v>421</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">0</f>
@@ -6607,7 +6748,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>413</v>
+        <v>422</v>
       </c>
       <c r="C9" s="31" t="n">
         <f aca="false">C6/C7</f>
@@ -6622,12 +6763,12 @@
         <v>1.29464235422864</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>414</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>415</v>
+        <v>424</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -6637,7 +6778,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>416</v>
+        <v>425</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">Tricity_Recon!C46</f>
@@ -6655,7 +6796,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>417</v>
+        <v>426</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">Tricity_Recon!C47</f>
@@ -6673,7 +6814,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>418</v>
+        <v>427</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -6683,7 +6824,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>419</v>
+        <v>428</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">TAM_India!C31*Assumptions!$C$34/Assumptions!$C$33*Assumptions!$C$54</f>
@@ -6698,12 +6839,12 @@
         <v>10141.9872254916</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>420</v>
+        <v>429</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>421</v>
+        <v>430</v>
       </c>
       <c r="C17" s="25" t="n">
         <f aca="false">Assumptions!$C$68</f>
@@ -6721,7 +6862,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>422</v>
+        <v>431</v>
       </c>
       <c r="C18" s="24" t="n">
         <f aca="false">C16*C17</f>
@@ -6739,7 +6880,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>423</v>
+        <v>432</v>
       </c>
       <c r="C19" s="24" t="n">
         <f aca="false">Tricity_Recon!C48</f>
@@ -6754,12 +6895,12 @@
         <v>263.76</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>424</v>
+        <v>433</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>425</v>
+        <v>434</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">MAX(0,C18-C19)</f>
@@ -6777,7 +6918,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>426</v>
+        <v>435</v>
       </c>
       <c r="C21" s="31" t="n">
         <f aca="false">C20*Assumptions!$C$56/10000000</f>
@@ -6792,12 +6933,12 @@
         <v>10.5878246705899</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>427</v>
+        <v>436</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>428</v>
+        <v>437</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -6807,7 +6948,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>429</v>
+        <v>438</v>
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">C16-C18</f>
@@ -6825,7 +6966,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>430</v>
+        <v>439</v>
       </c>
       <c r="C25" s="25" t="n">
         <f aca="false">Assumptions!$C$69</f>
@@ -6843,7 +6984,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>431</v>
+        <v>440</v>
       </c>
       <c r="C26" s="24" t="n">
         <f aca="false">C24*C25</f>
@@ -6861,7 +7002,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>432</v>
+        <v>441</v>
       </c>
       <c r="C27" s="31" t="n">
         <f aca="false">C26*Assumptions!$C$70/10000000</f>
@@ -6876,12 +7017,12 @@
         <v>5.84178464188316</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>433</v>
+        <v>442</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>434</v>
+        <v>443</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -6891,7 +7032,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>435</v>
+        <v>444</v>
       </c>
       <c r="C30" s="24" t="n">
         <f aca="false">Assumptions!$C$71+Assumptions!$C$72</f>
@@ -6906,12 +7047,12 @@
         <v>5300</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>436</v>
+        <v>445</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>437</v>
+        <v>446</v>
       </c>
       <c r="C31" s="24" t="n">
         <f aca="false">C30*Assumptions!$C$73</f>
@@ -6929,7 +7070,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">C31*Assumptions!$C$74/10000000</f>
@@ -6944,12 +7085,12 @@
         <v>2.544</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>439</v>
+        <v>448</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>440</v>
+        <v>449</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -6959,7 +7100,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>441</v>
+        <v>450</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">TAM_India!C33*Assumptions!$C$75</f>
@@ -6974,12 +7115,12 @@
         <v>54</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>443</v>
+        <v>452</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -6989,7 +7130,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>444</v>
+        <v>453</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">C13+C21+C27+C32</f>
@@ -7004,12 +7145,12 @@
         <v>24.2488093124731</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>446</v>
+        <v>455</v>
       </c>
       <c r="C39" s="22" t="n">
         <f aca="false">C35</f>
@@ -7024,12 +7165,12 @@
         <v>54</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>447</v>
+        <v>456</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>448</v>
+        <v>457</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">C38+C39</f>
@@ -7047,7 +7188,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>449</v>
+        <v>458</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">C12+C20+C26</f>
@@ -7065,7 +7206,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
-        <v>450</v>
+        <v>459</v>
       </c>
       <c r="C42" s="25" t="n">
         <f aca="false">C40/TAM_India!C34</f>
@@ -7083,7 +7224,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>451</v>
+        <v>460</v>
       </c>
       <c r="C43" s="22" t="n">
         <f aca="false">C13+C16*Assumptions!$C$56/10000000</f>
@@ -7098,12 +7239,12 @@
         <v>66.1271233529496</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>452</v>
+        <v>461</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="23" t="s">
-        <v>453</v>
+        <v>462</v>
       </c>
       <c r="C44" s="22" t="n">
         <f aca="false">TAM_India!C38*Assumptions!$C$56/TAM_India!C13</f>
@@ -7118,7 +7259,7 @@
         <v>57.834</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>454</v>
+        <v>463</v>
       </c>
     </row>
   </sheetData>
@@ -7137,7 +7278,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -7148,37 +7289,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>455</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>456</v>
+        <v>465</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>457</v>
+        <v>466</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>458</v>
+        <v>467</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>459</v>
+        <v>468</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -7188,359 +7329,445 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>460</v>
+        <v>469</v>
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">Assumptions!$C$78*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
+        <v>0.230218</v>
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">Assumptions!$D$78*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
+        <v>0.848066</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">Assumptions!$E$78*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
+        <v>1.233926</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>461</v>
+        <v>470</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>462</v>
+        <v>471</v>
       </c>
       <c r="C7" s="37" t="n">
         <f aca="false">IFERROR(C6/SAM_North!C13,0)</f>
-        <v>0</v>
+        <v>0.158469075183095</v>
       </c>
       <c r="D7" s="37" t="n">
         <f aca="false">IFERROR(D6/SAM_North!D13,0)</f>
-        <v>0</v>
+        <v>0.259543330317605</v>
       </c>
       <c r="E7" s="37" t="n">
         <f aca="false">IFERROR(E6/SAM_North!E13,0)</f>
-        <v>0</v>
+        <v>0.233910752198969</v>
       </c>
       <c r="F7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>463</v>
+        <v>472</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">Assumptions!$C$79*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
+        <v>0.04012</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">Assumptions!$D$79*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
+        <v>0.293348</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">Assumptions!$E$79*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
+        <v>0.891608</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>464</v>
+        <v>473</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>465</v>
+        <v>474</v>
       </c>
       <c r="C9" s="37" t="n">
         <f aca="false">IFERROR(C8/SAM_North!C21,0)</f>
-        <v>0</v>
+        <v>0.266942300424136</v>
       </c>
       <c r="D9" s="37" t="n">
         <f aca="false">IFERROR(D8/SAM_North!D21,0)</f>
-        <v>0</v>
+        <v>0.151277776670061</v>
       </c>
       <c r="E9" s="37" t="n">
         <f aca="false">IFERROR(E8/SAM_North!E21,0)</f>
-        <v>0</v>
+        <v>0.0842106880062571</v>
       </c>
       <c r="F9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>466</v>
+        <v>475</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">Assumptions!$C$80*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
+        <v>0.054634</v>
       </c>
       <c r="D10" s="22" t="n">
         <f aca="false">Assumptions!$D$80*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
+        <v>0.29677</v>
       </c>
       <c r="E10" s="22" t="n">
         <f aca="false">Assumptions!$E$80*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
+        <v>0.58233</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>467</v>
+        <v>476</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>468</v>
+        <v>477</v>
       </c>
       <c r="C11" s="37" t="n">
         <f aca="false">IFERROR(C10/SAM_North!C27,0)</f>
-        <v>0</v>
+        <v>0.247296083749113</v>
       </c>
       <c r="D11" s="37" t="n">
         <f aca="false">IFERROR(D10/SAM_North!D27,0)</f>
-        <v>0</v>
+        <v>0.213777924530198</v>
       </c>
       <c r="E11" s="37" t="n">
         <f aca="false">IFERROR(E10/SAM_North!E27,0)</f>
-        <v>0</v>
+        <v>0.0996835788544714</v>
       </c>
       <c r="F11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>469</v>
+        <v>478</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">Assumptions!$C$81*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
+        <v>0.068912</v>
       </c>
       <c r="D12" s="22" t="n">
         <f aca="false">Assumptions!$D$81*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
+        <v>0.319308</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">Assumptions!$E$81*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
+        <v>0.72157</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>470</v>
+        <v>479</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>471</v>
+        <v>480</v>
       </c>
       <c r="C13" s="37" t="n">
         <f aca="false">IFERROR(C12/SAM_North!C32,0)</f>
-        <v>0</v>
+        <v>0.153821428571429</v>
       </c>
       <c r="D13" s="37" t="n">
         <f aca="false">IFERROR(D12/SAM_North!D32,0)</f>
-        <v>0</v>
+        <v>0.26609</v>
       </c>
       <c r="E13" s="37" t="n">
         <f aca="false">IFERROR(E12/SAM_North!E32,0)</f>
-        <v>0</v>
+        <v>0.283636006289308</v>
       </c>
       <c r="F13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>472</v>
+        <v>481</v>
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">Assumptions!$C$82*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
+        <v>0.014986</v>
       </c>
       <c r="D14" s="22" t="n">
         <f aca="false">Assumptions!$D$82*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
+        <v>0.134874</v>
       </c>
       <c r="E14" s="22" t="n">
         <f aca="false">Assumptions!$E$82*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
+        <v>0.399784</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>473</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>474</v>
+        <v>483</v>
       </c>
       <c r="C15" s="37" t="n">
         <f aca="false">IFERROR(C14/SAM_North!C35,0)</f>
-        <v>0</v>
+        <v>0.0199813333333333</v>
       </c>
       <c r="D15" s="37" t="n">
         <f aca="false">IFERROR(D14/SAM_North!D35,0)</f>
-        <v>0</v>
+        <v>0.0171268571428571</v>
       </c>
       <c r="E15" s="37" t="n">
         <f aca="false">IFERROR(E14/SAM_North!E35,0)</f>
-        <v>0</v>
+        <v>0.00740340740740741</v>
       </c>
       <c r="F15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="C16" s="31" t="n">
-        <f aca="false">C6+C8+C10+C12+C14</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="31" t="n">
-        <f aca="false">D6+D8+D10+D12+D14</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="31" t="n">
-        <f aca="false">E6+E8+E10+E12+E14</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="2"/>
+      <c r="A16" s="7" t="s">
+        <v>484</v>
+      </c>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>476</v>
+        <v>485</v>
       </c>
       <c r="C17" s="37" t="n">
-        <f aca="false">(C16-C14)/SAM_North!C38</f>
-        <v>0</v>
+        <f aca="false">Assumptions!$C$84/SAM_North!C12</f>
+        <v>0.0693850297476997</v>
       </c>
       <c r="D17" s="37" t="n">
-        <f aca="false">(D16-D14)/SAM_North!D38</f>
-        <v>0</v>
+        <f aca="false">Assumptions!$D$84/SAM_North!D12</f>
+        <v>0.12931780571996</v>
       </c>
       <c r="E17" s="37" t="n">
-        <f aca="false">(E16-E14)/SAM_North!E38</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="2"/>
+        <f aca="false">Assumptions!$E$84/SAM_North!E12</f>
+        <v>0.11089626933576</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
-        <v>477</v>
-      </c>
-      <c r="C18" s="25" t="n">
-        <f aca="false">C16/SAM_North!C40</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="25" t="n">
-        <f aca="false">D16/SAM_North!D40</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="25" t="n">
-        <f aca="false">E16/SAM_North!E40</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="2"/>
+      <c r="A18" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="C18" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$C$85/(SAM_North!C20+Tricity_Recon!C48),0)</f>
+        <v>0.0602918299143058</v>
+      </c>
+      <c r="D18" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$D$85/(SAM_North!D20+Tricity_Recon!D48),0)</f>
+        <v>0.0656381860807753</v>
+      </c>
+      <c r="E18" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$E$85/(SAM_North!E20+Tricity_Recon!E48),0)</f>
+        <v>0.0468350027897985</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
-        <v>478</v>
-      </c>
-      <c r="C19" s="33" t="n">
-        <f aca="false">C16/TAM_India!C34</f>
-        <v>0</v>
-      </c>
-      <c r="D19" s="33" t="n">
-        <f aca="false">D16/TAM_India!D34</f>
-        <v>0</v>
-      </c>
-      <c r="E19" s="33" t="n">
-        <f aca="false">E16/TAM_India!E34</f>
-        <v>0</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>479</v>
-      </c>
+      <c r="A19" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="C19" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$C$86/SAM_North!C26,0)</f>
+        <v>0.144845237031365</v>
+      </c>
+      <c r="D19" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$D$86/SAM_North!D26,0)</f>
+        <v>0.126061046577433</v>
+      </c>
+      <c r="E19" s="37" t="n">
+        <f aca="false">IFERROR(Assumptions!$E$86/SAM_North!E26,0)</f>
+        <v>0.0553597949642574</v>
+      </c>
+      <c r="F19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>480</v>
-      </c>
-      <c r="C20" s="22" t="n">
-        <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="D20" s="22" t="n">
-        <f aca="false">Assumptions!$D$83*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="E20" s="22" t="n">
-        <f aca="false">Assumptions!$E$83*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>481</v>
-      </c>
+        <v>490</v>
+      </c>
+      <c r="C20" s="25" t="n">
+        <f aca="false">Assumptions!$C$84/Tricity_Recon!C15</f>
+        <v>0.0566666666666667</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <f aca="false">Assumptions!$D$84/Tricity_Recon!D15</f>
+        <v>0.0747611464968153</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <f aca="false">Assumptions!$E$84/Tricity_Recon!E15</f>
+        <v>0.04375</v>
+      </c>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="C21" s="31" t="n">
+        <f aca="false">C6+C8+C10+C12+C14</f>
+        <v>0.40887</v>
+      </c>
+      <c r="D21" s="31" t="n">
+        <f aca="false">D6+D8+D10+D12+D14</f>
+        <v>1.892366</v>
+      </c>
+      <c r="E21" s="31" t="n">
+        <f aca="false">E6+E8+E10+E12+E14</f>
+        <v>3.829218</v>
+      </c>
+      <c r="F21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="s">
-        <v>482</v>
-      </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="A22" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="C22" s="37" t="n">
+        <f aca="false">(C21-C14)/SAM_North!C38</f>
+        <v>0.173365730000161</v>
+      </c>
+      <c r="D22" s="37" t="n">
+        <f aca="false">(D21-D14)/SAM_North!D38</f>
+        <v>0.225467412124093</v>
+      </c>
+      <c r="E22" s="37" t="n">
+        <f aca="false">(E21-E14)/SAM_North!E38</f>
+        <v>0.141426902896876</v>
+      </c>
+      <c r="F22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>483</v>
-      </c>
-      <c r="C23" s="22" t="n">
-        <f aca="false">Assumptions!$C$84*(1+Assumptions!$C$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="22" t="n">
-        <f aca="false">Assumptions!$D$84*(1+Assumptions!$D$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="22" t="n">
-        <f aca="false">Assumptions!$E$84*(1+Assumptions!$E$76)/100</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>484</v>
-      </c>
+        <v>493</v>
+      </c>
+      <c r="C23" s="25" t="n">
+        <f aca="false">C21/SAM_North!C40</f>
+        <v>0.135298574890674</v>
+      </c>
+      <c r="D23" s="25" t="n">
+        <f aca="false">D21/SAM_North!D40</f>
+        <v>0.12076452979223</v>
+      </c>
+      <c r="E23" s="25" t="n">
+        <f aca="false">E21/SAM_North!E40</f>
+        <v>0.0489364379297924</v>
+      </c>
+      <c r="F23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>485</v>
-      </c>
-      <c r="C24" s="37" t="n">
-        <f aca="false">C23/SAM_North!C13</f>
-        <v>0</v>
-      </c>
-      <c r="D24" s="37" t="n">
-        <f aca="false">D23/SAM_North!D13</f>
-        <v>0</v>
-      </c>
-      <c r="E24" s="37" t="n">
-        <f aca="false">E23/SAM_North!E13</f>
-        <v>0</v>
+      <c r="A24" s="23" t="s">
+        <v>494</v>
+      </c>
+      <c r="C24" s="33" t="n">
+        <f aca="false">C21/TAM_India!C34</f>
+        <v>0.00493223559214693</v>
+      </c>
+      <c r="D24" s="33" t="n">
+        <f aca="false">D21/TAM_India!D34</f>
+        <v>0.00461276690394848</v>
+      </c>
+      <c r="E24" s="33" t="n">
+        <f aca="false">E21/TAM_India!E34</f>
+        <v>0.0025640940136601</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>486</v>
+        <v>495</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>487</v>
-      </c>
-      <c r="C25" s="35" t="n">
-        <f aca="false">IFERROR(C16/C23,0)</f>
-        <v>0</v>
-      </c>
-      <c r="D25" s="35" t="n">
-        <f aca="false">IFERROR(D16/D23,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E25" s="35" t="n">
-        <f aca="false">IFERROR(E16/E23,0)</f>
-        <v>0</v>
-      </c>
-      <c r="F25" s="2"/>
+        <v>496</v>
+      </c>
+      <c r="C25" s="22" t="n">
+        <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$76)/100</f>
+        <v>0.0236</v>
+      </c>
+      <c r="D25" s="22" t="n">
+        <f aca="false">Assumptions!$D$83*(1+Assumptions!$D$76)/100</f>
+        <v>0.07729</v>
+      </c>
+      <c r="E25" s="22" t="n">
+        <f aca="false">Assumptions!$E$83*(1+Assumptions!$E$76)/100</f>
+        <v>0.119534</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>497</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>488</v>
+      <c r="A27" s="7" t="s">
+        <v>498</v>
+      </c>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="s">
+        <v>499</v>
+      </c>
+      <c r="C28" s="22" t="n">
+        <f aca="false">Assumptions!$C$87*(1+Assumptions!$C$76)/100</f>
+        <v>0.079178</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <f aca="false">Assumptions!$D$87*(1+Assumptions!$D$76)/100</f>
+        <v>0.195998</v>
+      </c>
+      <c r="E28" s="22" t="n">
+        <f aca="false">Assumptions!$E$87*(1+Assumptions!$E$76)/100</f>
+        <v>0.294056</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="C29" s="37" t="n">
+        <f aca="false">C28/SAM_North!C13</f>
+        <v>0.0545016655293985</v>
+      </c>
+      <c r="D29" s="37" t="n">
+        <f aca="false">D28/SAM_North!D13</f>
+        <v>0.0599835079529068</v>
+      </c>
+      <c r="E29" s="37" t="n">
+        <f aca="false">E28/SAM_North!E13</f>
+        <v>0.0557430997876858</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="23" t="s">
+        <v>503</v>
+      </c>
+      <c r="C30" s="35" t="n">
+        <f aca="false">IFERROR(C21/C28,0)</f>
+        <v>5.16393442622951</v>
+      </c>
+      <c r="D30" s="35" t="n">
+        <f aca="false">IFERROR(D21/D28,0)</f>
+        <v>9.65502709211319</v>
+      </c>
+      <c r="E30" s="35" t="n">
+        <f aca="false">IFERROR(E21/E28,0)</f>
+        <v>13.0220706260032</v>
+      </c>
+      <c r="F30" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -7559,7 +7786,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -7571,17 +7798,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>489</v>
+        <v>505</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>490</v>
+        <v>506</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>491</v>
+        <v>507</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6" t="s">
@@ -7594,15 +7821,15 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>492</v>
+        <v>508</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>493</v>
+        <v>509</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>494</v>
+        <v>510</v>
       </c>
       <c r="C5" s="29" t="n">
         <f aca="false">TAM_India!C30</f>
@@ -7621,12 +7848,12 @@
         <v>387.7453125</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>495</v>
+        <v>511</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>496</v>
+        <v>512</v>
       </c>
       <c r="C6" s="29" t="n">
         <f aca="false">TAM_India!C33</f>
@@ -7645,12 +7872,12 @@
         <v>22.5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>497</v>
+        <v>513</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>498</v>
+        <v>514</v>
       </c>
       <c r="C7" s="29" t="n">
         <f aca="false">TAM_India!C38</f>
@@ -7669,12 +7896,12 @@
         <v>29.66251640625</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>499</v>
+        <v>515</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>500</v>
+        <v>516</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">SAM_North!C40</f>
@@ -7693,12 +7920,12 @@
         <v>15.6698825661453</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>501</v>
+        <v>517</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>502</v>
+        <v>518</v>
       </c>
       <c r="C9" s="22" t="n">
         <f aca="false">SAM_North!C38</f>
@@ -7717,12 +7944,12 @@
         <v>7.79488256614533</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>445</v>
+        <v>454</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>503</v>
+        <v>519</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">SAM_North!C13</f>
@@ -7741,12 +7968,12 @@
         <v>3.26753147138174</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>504</v>
+        <v>520</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>505</v>
+        <v>521</v>
       </c>
       <c r="C11" s="22" t="n">
         <f aca="false">SAM_North!C21</f>
@@ -7765,12 +7992,12 @@
         <v>1.93913479201771</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>506</v>
+        <v>522</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>507</v>
+        <v>523</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">SAM_North!C27</f>
@@ -7792,7 +8019,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>508</v>
+        <v>524</v>
       </c>
       <c r="C13" s="22" t="n">
         <f aca="false">SAM_North!C32</f>
@@ -7811,12 +8038,12 @@
         <v>1.2</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>509</v>
+        <v>525</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>510</v>
+        <v>526</v>
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">SAM_North!C35</f>
@@ -7838,143 +8065,167 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>511</v>
+        <v>527</v>
       </c>
       <c r="C15" s="22" t="n">
-        <f aca="false">SOM_PNA!C16</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!C21</f>
+        <v>0.40887</v>
       </c>
       <c r="D15" s="22" t="n">
-        <f aca="false">SOM_PNA!D16</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!D21</f>
+        <v>1.892366</v>
       </c>
       <c r="E15" s="22" t="n">
-        <f aca="false">SOM_PNA!E16</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!E21</f>
+        <v>3.829218</v>
       </c>
       <c r="F15" s="21" t="n">
         <f aca="false">INDEX(C15:E15,Assumptions!$C$4)</f>
-        <v>0</v>
+        <v>1.892366</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>512</v>
+        <v>528</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>513</v>
+        <v>529</v>
       </c>
       <c r="C16" s="25" t="n">
-        <f aca="false">SOM_PNA!C17</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!C22</f>
+        <v>0.173365730000161</v>
       </c>
       <c r="D16" s="25" t="n">
-        <f aca="false">SOM_PNA!D17</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!D22</f>
+        <v>0.225467412124093</v>
       </c>
       <c r="E16" s="25" t="n">
-        <f aca="false">SOM_PNA!E17</f>
-        <v>0</v>
+        <f aca="false">SOM_PNA!E22</f>
+        <v>0.141426902896876</v>
       </c>
       <c r="F16" s="13" t="n">
         <f aca="false">INDEX(C16:E16,Assumptions!$C$4)</f>
-        <v>0</v>
+        <v>0.225467412124093</v>
       </c>
       <c r="G16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>514</v>
-      </c>
-      <c r="C17" s="33" t="n">
-        <f aca="false">SOM_PNA!C19</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="33" t="n">
-        <f aca="false">SOM_PNA!D19</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="33" t="n">
-        <f aca="false">SOM_PNA!E19</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="19" t="n">
+        <v>530</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <f aca="false">SOM_PNA!C17</f>
+        <v>0.0693850297476997</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <f aca="false">SOM_PNA!D17</f>
+        <v>0.12931780571996</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <f aca="false">SOM_PNA!E17</f>
+        <v>0.11089626933576</v>
+      </c>
+      <c r="F17" s="13" t="n">
         <f aca="false">INDEX(C17:E17,Assumptions!$C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="2"/>
+        <v>0.12931780571996</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>531</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>515</v>
-      </c>
-      <c r="C18" s="22" t="n">
-        <f aca="false">SOM_PNA!C23</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="22" t="n">
-        <f aca="false">SOM_PNA!D23</f>
-        <v>0</v>
-      </c>
-      <c r="E18" s="22" t="n">
-        <f aca="false">SOM_PNA!E23</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="21" t="n">
+      <c r="A18" s="0" t="s">
+        <v>532</v>
+      </c>
+      <c r="C18" s="33" t="n">
+        <f aca="false">SOM_PNA!C24</f>
+        <v>0.00493223559214693</v>
+      </c>
+      <c r="D18" s="33" t="n">
+        <f aca="false">SOM_PNA!D24</f>
+        <v>0.00461276690394848</v>
+      </c>
+      <c r="E18" s="33" t="n">
+        <f aca="false">SOM_PNA!E24</f>
+        <v>0.0025640940136601</v>
+      </c>
+      <c r="F18" s="19" t="n">
         <f aca="false">INDEX(C18:E18,Assumptions!$C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>516</v>
-      </c>
+        <v>0.00461276690394848</v>
+      </c>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>517</v>
-      </c>
-      <c r="C19" s="24" t="n">
+        <v>533</v>
+      </c>
+      <c r="C19" s="22" t="n">
+        <f aca="false">SOM_PNA!C28</f>
+        <v>0.079178</v>
+      </c>
+      <c r="D19" s="22" t="n">
+        <f aca="false">SOM_PNA!D28</f>
+        <v>0.195998</v>
+      </c>
+      <c r="E19" s="22" t="n">
+        <f aca="false">SOM_PNA!E28</f>
+        <v>0.294056</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <f aca="false">INDEX(C19:E19,Assumptions!$C$4)</f>
+        <v>0.195998</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>535</v>
+      </c>
+      <c r="C20" s="24" t="n">
         <f aca="false">TAM_India!C31</f>
         <v>20100</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D20" s="24" t="n">
         <f aca="false">TAM_India!D31</f>
         <v>56812.5</v>
       </c>
-      <c r="E19" s="24" t="n">
+      <c r="E20" s="24" t="n">
         <f aca="false">TAM_India!E31</f>
         <v>126000</v>
       </c>
-      <c r="F19" s="11" t="n">
-        <f aca="false">INDEX(C19:E19,Assumptions!$C$4)</f>
+      <c r="F20" s="11" t="n">
+        <f aca="false">INDEX(C20:E20,Assumptions!$C$4)</f>
         <v>56812.5</v>
       </c>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>518</v>
-      </c>
-      <c r="C20" s="24" t="n">
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="C21" s="24" t="n">
         <f aca="false">Tricity_Recon!C46</f>
         <v>484.254314254494</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D21" s="24" t="n">
         <f aca="false">Tricity_Recon!D46</f>
         <v>726.118104751498</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E21" s="24" t="n">
         <f aca="false">Tricity_Recon!E46</f>
         <v>879.2</v>
       </c>
-      <c r="F20" s="11" t="n">
-        <f aca="false">INDEX(C20:E20,Assumptions!$C$4)</f>
+      <c r="F21" s="11" t="n">
+        <f aca="false">INDEX(C21:E21,Assumptions!$C$4)</f>
         <v>726.118104751498</v>
       </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
-        <v>519</v>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>537</v>
       </c>
     </row>
   </sheetData>
@@ -8005,29 +8256,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>520</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>521</v>
+        <v>539</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>522</v>
+        <v>540</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>523</v>
+        <v>541</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>524</v>
+        <v>542</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>525</v>
+        <v>543</v>
       </c>
       <c r="B5" s="29" t="n">
         <v>276999</v>
@@ -8036,15 +8287,15 @@
         <v>105</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>526</v>
+        <v>544</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>527</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>528</v>
+        <v>546</v>
       </c>
       <c r="B6" s="29" t="n">
         <v>76141</v>
@@ -8053,49 +8304,49 @@
         <v>105</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>526</v>
+        <v>544</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>529</v>
+        <v>547</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>530</v>
+        <v>548</v>
       </c>
       <c r="B7" s="29" t="n">
         <v>1.52</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>531</v>
+        <v>549</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>532</v>
+        <v>550</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>533</v>
+        <v>551</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>534</v>
+        <v>552</v>
       </c>
       <c r="B8" s="29" t="n">
         <v>12.6</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>531</v>
+        <v>549</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>535</v>
+        <v>553</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>536</v>
+        <v>554</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>537</v>
+        <v>555</v>
       </c>
       <c r="B9" s="29" t="n">
         <v>2880</v>
@@ -8104,15 +8355,15 @@
         <v>105</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>538</v>
+        <v>556</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>539</v>
+        <v>557</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>540</v>
+        <v>558</v>
       </c>
       <c r="B10" s="29" t="n">
         <v>650000</v>
@@ -8121,15 +8372,15 @@
         <v>105</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>541</v>
+        <v>559</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>542</v>
+        <v>560</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>543</v>
+        <v>561</v>
       </c>
       <c r="B11" s="29" t="n">
         <f aca="false">TAM_India!D36</f>
@@ -8139,15 +8390,15 @@
         <v>105</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>544</v>
+        <v>562</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>545</v>
+        <v>563</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>546</v>
+        <v>564</v>
       </c>
       <c r="B13" s="29" t="n">
         <f aca="false">TAM_India!D30</f>
@@ -8180,23 +8431,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>547</v>
+        <v>565</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>548</v>
+        <v>566</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>549</v>
+        <v>567</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>550</v>
+        <v>568</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>551</v>
+        <v>569</v>
       </c>
       <c r="B5" s="38" t="b">
         <f aca="false">ABS(TAM_India!D14-522.1)&lt;1</f>
@@ -8205,7 +8456,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>552</v>
+        <v>570</v>
       </c>
       <c r="B6" s="38" t="b">
         <f aca="false">ABS(TAM_India!D30-387.7)&lt;1</f>
@@ -8214,7 +8465,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>553</v>
+        <v>571</v>
       </c>
       <c r="B7" s="38" t="b">
         <f aca="false">ABS(Tricity_Recon!D16-5.65)&lt;0.1</f>
@@ -8223,7 +8474,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>554</v>
+        <v>572</v>
       </c>
       <c r="B8" s="38" t="b">
         <f aca="false">AND(Tricity_Recon!D46&gt;=Tricity_Recon!D28,Tricity_Recon!D46&lt;=Tricity_Recon!D34)</f>
@@ -8232,7 +8483,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>555</v>
+        <v>573</v>
       </c>
       <c r="B9" s="38" t="b">
         <f aca="false">AND(Tricity_Recon!C47&lt;=Tricity_Recon!D47,Tricity_Recon!D47&lt;=Tricity_Recon!E47)</f>
@@ -8241,7 +8492,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>556</v>
+        <v>574</v>
       </c>
       <c r="B10" s="38" t="b">
         <f aca="false">AND(SAM_North!C40&lt;TAM_India!C34,SAM_North!D40&lt;TAM_India!D34,SAM_North!E40&lt;TAM_India!E34)</f>
@@ -8250,25 +8501,25 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>557</v>
+        <v>575</v>
       </c>
       <c r="B11" s="38" t="b">
-        <f aca="false">AND(SOM_PNA!C16&lt;SAM_North!C40,SOM_PNA!D16&lt;SAM_North!D40,SOM_PNA!E16&lt;SAM_North!E40)</f>
+        <f aca="false">AND(SOM_PNA!C21&lt;SAM_North!C40,SOM_PNA!D21&lt;SAM_North!D40,SOM_PNA!E21&lt;SAM_North!E40)</f>
         <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>558</v>
+        <v>576</v>
       </c>
       <c r="B12" s="38" t="b">
-        <f aca="false">SOM_PNA!D7&lt;=0.25</f>
+        <f aca="false">SOM_PNA!D17&lt;=0.25</f>
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>559</v>
+        <v>577</v>
       </c>
       <c r="B13" s="38" t="b">
         <f aca="false">ABS(Tricity_Recon!D12/Tricity_Recon!D10-1)&lt;0.1</f>
@@ -8277,7 +8528,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>560</v>
+        <v>578</v>
       </c>
       <c r="B15" s="38" t="b">
         <f aca="false">AND(B5:B13)</f>

</xml_diff>

<commit_message>
Add economics models: market sizing, business forecast, funnel economics
Auditable openpyxl workbooks with formulas, recalculated in LibreOffice;
assumptions register consolidated and tricity/India sizing reconciled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K2weV5RtvDCshBNnABKa1E
</commit_message>
<xml_diff>
--- a/priyanka_nanda_academy/economics/market_sizing_model.xlsx
+++ b/priyanka_nanda_academy/economics/market_sizing_model.xlsx
@@ -4555,7 +4555,7 @@
         <v>19.51</v>
       </c>
       <c r="D78" s="16" t="n">
-        <v>71.87</v>
+        <v>71.88</v>
       </c>
       <c r="E78" s="16" t="n">
         <v>104.57</v>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="I78" s="17" t="n">
         <f aca="false">INDEX(C78:E78,$C$4)</f>
-        <v>71.87</v>
+        <v>71.88</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7337,7 +7337,7 @@
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">Assumptions!$D$78*(1+Assumptions!$D$76)/100</f>
-        <v>0.848066</v>
+        <v>0.848184</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">Assumptions!$E$78*(1+Assumptions!$E$76)/100</f>
@@ -7357,7 +7357,7 @@
       </c>
       <c r="D7" s="37" t="n">
         <f aca="false">IFERROR(D6/SAM_North!D13,0)</f>
-        <v>0.259543330317605</v>
+        <v>0.259579443206198</v>
       </c>
       <c r="E7" s="37" t="n">
         <f aca="false">IFERROR(E6/SAM_North!E13,0)</f>
@@ -7613,7 +7613,7 @@
       </c>
       <c r="D21" s="31" t="n">
         <f aca="false">D6+D8+D10+D12+D14</f>
-        <v>1.892366</v>
+        <v>1.892484</v>
       </c>
       <c r="E21" s="31" t="n">
         <f aca="false">E6+E8+E10+E12+E14</f>
@@ -7631,7 +7631,7 @@
       </c>
       <c r="D22" s="37" t="n">
         <f aca="false">(D21-D14)/SAM_North!D38</f>
-        <v>0.225467412124093</v>
+        <v>0.22548255026107</v>
       </c>
       <c r="E22" s="37" t="n">
         <f aca="false">(E21-E14)/SAM_North!E38</f>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="D23" s="25" t="n">
         <f aca="false">D21/SAM_North!D40</f>
-        <v>0.12076452979223</v>
+        <v>0.120772060161363</v>
       </c>
       <c r="E23" s="25" t="n">
         <f aca="false">E21/SAM_North!E40</f>
@@ -7667,7 +7667,7 @@
       </c>
       <c r="D24" s="33" t="n">
         <f aca="false">D21/TAM_India!D34</f>
-        <v>0.00461276690394848</v>
+        <v>0.00461305453672917</v>
       </c>
       <c r="E24" s="33" t="n">
         <f aca="false">E21/TAM_India!E34</f>
@@ -7757,7 +7757,7 @@
       </c>
       <c r="D30" s="35" t="n">
         <f aca="false">IFERROR(D21/D28,0)</f>
-        <v>9.65502709211319</v>
+        <v>9.65562913907285</v>
       </c>
       <c r="E30" s="35" t="n">
         <f aca="false">IFERROR(E21/E28,0)</f>
@@ -8073,7 +8073,7 @@
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">SOM_PNA!D21</f>
-        <v>1.892366</v>
+        <v>1.892484</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">SOM_PNA!E21</f>
@@ -8081,7 +8081,7 @@
       </c>
       <c r="F15" s="21" t="n">
         <f aca="false">INDEX(C15:E15,Assumptions!$C$4)</f>
-        <v>1.892366</v>
+        <v>1.892484</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>528</v>
@@ -8097,7 +8097,7 @@
       </c>
       <c r="D16" s="25" t="n">
         <f aca="false">SOM_PNA!D22</f>
-        <v>0.225467412124093</v>
+        <v>0.22548255026107</v>
       </c>
       <c r="E16" s="25" t="n">
         <f aca="false">SOM_PNA!E22</f>
@@ -8105,7 +8105,7 @@
       </c>
       <c r="F16" s="13" t="n">
         <f aca="false">INDEX(C16:E16,Assumptions!$C$4)</f>
-        <v>0.225467412124093</v>
+        <v>0.22548255026107</v>
       </c>
       <c r="G16" s="2"/>
     </row>
@@ -8143,7 +8143,7 @@
       </c>
       <c r="D18" s="33" t="n">
         <f aca="false">SOM_PNA!D24</f>
-        <v>0.00461276690394848</v>
+        <v>0.00461305453672917</v>
       </c>
       <c r="E18" s="33" t="n">
         <f aca="false">SOM_PNA!E24</f>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="F18" s="19" t="n">
         <f aca="false">INDEX(C18:E18,Assumptions!$C$4)</f>
-        <v>0.00461276690394848</v>
+        <v>0.00461305453672917</v>
       </c>
       <c r="G18" s="2"/>
     </row>

</xml_diff>

<commit_message>
Align growth and martech files to canonical strategy vocabulary
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K2weV5RtvDCshBNnABKa1E
</commit_message>
<xml_diff>
--- a/priyanka_nanda_academy/economics/market_sizing_model.xlsx
+++ b/priyanka_nanda_academy/economics/market_sizing_model.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="588">
   <si>
     <t xml:space="preserve">PNA market sizing model - TAM / SAM / SOM with tricity-India reconciliation</t>
   </si>
@@ -825,6 +825,21 @@
     <t xml:space="preserve">Y3 incremental destination/hybrid learners</t>
   </si>
   <si>
+    <t xml:space="preserve">CA-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PNA paying students per year today (all courses) - founder 'under 60'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">students/yr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Founder 2026-10-16 (canonical CA-01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[FOUNDER]</t>
+  </si>
+  <si>
     <t xml:space="preserve">SOM-BASELINE</t>
   </si>
   <si>
@@ -1542,6 +1557,12 @@
     <t xml:space="preserve">Y3 SOM multiple of today</t>
   </si>
   <si>
+    <t xml:space="preserve">ILLUSTRATIVE: today's PNA share of tricity makeup-led learners (CA-01 / reconciled learners; Low = CA-01 low / market high, High = CA-01 high / market low)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All PNA students (career + short) over all makeup-led learners (incl. short-course). Not quoted as a fact until CA-01 is confirmed (V1)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Share tests: a single centre at &gt;25% of tricity, &gt;30% of CPD or &gt;5% of online would be a red flag (chandigarh_market_analysis §8.2; international_benchmarks §2).</t>
   </si>
   <si>
@@ -1633,6 +1654,12 @@
   </si>
   <si>
     <t xml:space="preserve">CA-01 x CA-02 assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Illustrative: today's PNA share of tricity makeup-led learners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CA-01 / reconciled learners; to confirm with V1</t>
   </si>
   <si>
     <t xml:space="preserve">Learners: India makeup-led paid learners</t>
@@ -2447,7 +2474,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M87"/>
+  <dimension ref="A1:M88"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -4821,26 +4848,56 @@
       <c r="B87" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="C87" s="16" t="n">
+      <c r="C87" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="D87" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="E87" s="9" t="n">
+        <v>60</v>
+      </c>
+      <c r="F87" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="H87" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="I87" s="11" t="n">
+        <f aca="false">INDEX(C87:E87,$C$4)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="C88" s="16" t="n">
         <v>6.71</v>
       </c>
-      <c r="D87" s="16" t="n">
+      <c r="D88" s="16" t="n">
         <v>16.61</v>
       </c>
-      <c r="E87" s="16" t="n">
+      <c r="E88" s="16" t="n">
         <v>24.92</v>
       </c>
-      <c r="F87" s="10" t="s">
+      <c r="F88" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="G87" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="H87" s="10" t="s">
+      <c r="G88" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="H88" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="I87" s="17" t="n">
-        <f aca="false">INDEX(C87:E87,$C$4)</f>
+      <c r="I88" s="17" t="n">
+        <f aca="false">INDEX(C88:E88,$C$4)</f>
         <v>16.61</v>
       </c>
     </row>
@@ -4877,20 +4934,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -4902,12 +4959,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -4917,10 +4974,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">Assumptions!$C$9</f>
@@ -4940,7 +4997,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">C6/Assumptions!$C$10</f>
@@ -4955,12 +5012,12 @@
         <v>525000</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C8" s="25" t="n">
         <f aca="false">C7/Assumptions!$C$29</f>
@@ -4975,12 +5032,12 @@
         <v>0.772485962826504</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C9" s="25" t="n">
         <f aca="false">Assumptions!$C$11</f>
@@ -5000,7 +5057,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C10" s="24" t="n">
         <f aca="false">C7*C9</f>
@@ -5015,12 +5072,12 @@
         <v>420000</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C11" s="25" t="n">
         <f aca="false">Assumptions!$C$12</f>
@@ -5040,7 +5097,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C12" s="26" t="n">
         <f aca="false">C10*C11</f>
@@ -5055,12 +5112,12 @@
         <v>147000</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C13" s="27" t="n">
         <f aca="false">Assumptions!$C$13*Assumptions!$C$14+Assumptions!$C$15*Assumptions!$C$16+Assumptions!$C$17*Assumptions!$C$18+Assumptions!$C$19*Assumptions!$C$20</f>
@@ -5075,12 +5132,12 @@
         <v>109000</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C14" s="28" t="n">
         <f aca="false">C12*C13/10000000</f>
@@ -5095,12 +5152,12 @@
         <v>1602.3</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C15" s="24" t="n">
         <f aca="false">C10-C12</f>
@@ -5115,12 +5172,12 @@
         <v>273000</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C16" s="29" t="n">
         <f aca="false">C15*Assumptions!$C$21/10000000</f>
@@ -5135,12 +5192,12 @@
         <v>491.4</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C17" s="29" t="n">
         <f aca="false">C14+C16</f>
@@ -5155,12 +5212,12 @@
         <v>2093.7</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -5170,7 +5227,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">Assumptions!$C$22</f>
@@ -5190,7 +5247,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="23" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C21" s="24" t="n">
         <f aca="false">Assumptions!$C$23</f>
@@ -5210,7 +5267,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C22" s="24" t="n">
         <f aca="false">C20*C21</f>
@@ -5225,12 +5282,12 @@
         <v>75000</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="C23" s="24" t="n">
         <f aca="false">C22*(1+Assumptions!$C$24)</f>
@@ -5245,12 +5302,12 @@
         <v>300000</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C24" s="26" t="n">
         <f aca="false">C23*Assumptions!$C$12</f>
@@ -5265,12 +5322,12 @@
         <v>105000</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C25" s="28" t="n">
         <f aca="false">C24*C13/10000000</f>
@@ -5285,12 +5342,12 @@
         <v>1144.5</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">(C23-C24)*Assumptions!$C$21/10000000</f>
@@ -5308,7 +5365,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="23" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C27" s="29" t="n">
         <f aca="false">C25+C26</f>
@@ -5326,7 +5383,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -5336,7 +5393,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C30" s="28" t="n">
         <f aca="false">AVERAGE(C14,C25)</f>
@@ -5351,12 +5408,12 @@
         <v>1373.4</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C31" s="26" t="n">
         <f aca="false">AVERAGE(C12,C24)</f>
@@ -5371,12 +5428,12 @@
         <v>126000</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">C31/Assumptions!$C$33</f>
@@ -5391,12 +5448,12 @@
         <v>0.565164346203531</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C33" s="29" t="n">
         <f aca="false">Assumptions!$C$25*Assumptions!$C$26/10000000</f>
@@ -5411,12 +5468,12 @@
         <v>120</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="C34" s="28" t="n">
         <f aca="false">C30+C33</f>
@@ -5434,7 +5491,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C35" s="29" t="n">
         <f aca="false">C30*10000000/Assumptions!$C$27/1000000</f>
@@ -5449,12 +5506,12 @@
         <v>156.068181818182</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="23" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C36" s="29" t="n">
         <f aca="false">AVERAGE(C17,C27)</f>
@@ -5469,12 +5526,12 @@
         <v>1794.6</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C37" s="25" t="n">
         <f aca="false">C30/Assumptions!$C$30</f>
@@ -5489,12 +5546,12 @@
         <v>0.0180375881588106</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C38" s="29" t="n">
         <f aca="false">C30*Assumptions!$C$28</f>
@@ -5509,12 +5566,12 @@
         <v>105.0651</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
     </row>
   </sheetData>
@@ -5544,20 +5601,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -5569,12 +5626,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -5584,7 +5641,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="22" t="n">
@@ -5600,12 +5657,12 @@
         <v>2.55601659751037</v>
       </c>
       <c r="F6" s="30" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="22" t="n">
@@ -5624,7 +5681,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" s="22" t="n">
@@ -5643,7 +5700,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" s="24" t="n">
@@ -5659,12 +5716,12 @@
         <v>471</v>
       </c>
       <c r="F9" s="30" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B10" s="2"/>
       <c r="C10" s="22" t="n">
@@ -5680,12 +5737,12 @@
         <v>2</v>
       </c>
       <c r="F10" s="30" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" s="10" t="n">
@@ -5704,7 +5761,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" s="31" t="n">
@@ -5720,12 +5777,12 @@
         <v>1.90293451735955</v>
       </c>
       <c r="F12" s="30" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -5735,7 +5792,7 @@
     </row>
     <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="23" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="24" t="n">
@@ -5751,12 +5808,12 @@
         <v>2228.57142857143</v>
       </c>
       <c r="F15" s="30" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="31" t="n">
@@ -5772,12 +5829,12 @@
         <v>13.3714285714286</v>
       </c>
       <c r="F16" s="30" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="29" t="n">
@@ -5793,12 +5850,12 @@
         <v>1373.4</v>
       </c>
       <c r="F17" s="30" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="32" t="n">
@@ -5814,12 +5871,12 @@
         <v>0.00973600449354054</v>
       </c>
       <c r="F18" s="30" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="33" t="n">
@@ -5835,12 +5892,12 @@
         <v>0.00233242428591933</v>
       </c>
       <c r="F19" s="30" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -5850,7 +5907,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="23" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="24" t="n">
@@ -5866,12 +5923,12 @@
         <v>126000</v>
       </c>
       <c r="F22" s="30" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="33" t="n">
@@ -5890,7 +5947,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B24" s="2"/>
       <c r="C24" s="22" t="n">
@@ -5906,12 +5963,12 @@
         <v>2.28</v>
       </c>
       <c r="F24" s="30" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="22" t="n">
@@ -5927,12 +5984,12 @@
         <v>1.83188405797101</v>
       </c>
       <c r="F25" s="30" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B26" s="2"/>
       <c r="C26" s="22" t="n">
@@ -5948,12 +6005,12 @@
         <v>1.42857142857143</v>
       </c>
       <c r="F26" s="30" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="32" t="n">
@@ -5972,7 +6029,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="B28" s="2"/>
       <c r="C28" s="26" t="n">
@@ -5991,7 +6048,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="22" t="n">
@@ -6007,12 +6064,12 @@
         <v>10.5211724839461</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="B31" s="8"/>
       <c r="C31" s="8"/>
@@ -6022,7 +6079,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="23" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="B32" s="2"/>
       <c r="C32" s="24" t="n">
@@ -6041,7 +6098,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="23" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="B33" s="2"/>
       <c r="C33" s="25" t="n">
@@ -6057,12 +6114,12 @@
         <v>0.8</v>
       </c>
       <c r="F33" s="30" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="B34" s="2"/>
       <c r="C34" s="26" t="n">
@@ -6081,7 +6138,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="23" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="B35" s="2"/>
       <c r="C35" s="22" t="n">
@@ -6100,7 +6157,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -6110,7 +6167,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B38" s="2"/>
       <c r="C38" s="24" t="n">
@@ -6126,12 +6183,12 @@
         <v>420</v>
       </c>
       <c r="F38" s="30" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="B39" s="2"/>
       <c r="C39" s="24" t="n">
@@ -6147,12 +6204,12 @@
         <v>300</v>
       </c>
       <c r="F39" s="30" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="23" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B40" s="2"/>
       <c r="C40" s="24" t="n">
@@ -6168,12 +6225,12 @@
         <v>320</v>
       </c>
       <c r="F40" s="30" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="24" t="n">
@@ -6189,12 +6246,12 @@
         <v>133.2</v>
       </c>
       <c r="F41" s="30" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B42" s="2"/>
       <c r="C42" s="26" t="n">
@@ -6213,7 +6270,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="B43" s="2"/>
       <c r="C43" s="22" t="n">
@@ -6232,7 +6289,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -6242,7 +6299,7 @@
     </row>
     <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="B46" s="2"/>
       <c r="C46" s="26" t="n">
@@ -6258,12 +6315,12 @@
         <v>879.2</v>
       </c>
       <c r="F46" s="30" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="B47" s="2"/>
       <c r="C47" s="31" t="n">
@@ -6279,12 +6336,12 @@
         <v>5.2752</v>
       </c>
       <c r="F47" s="30" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="23" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="B48" s="2"/>
       <c r="C48" s="24" t="n">
@@ -6303,7 +6360,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="3" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
       <c r="B49" s="2"/>
       <c r="C49" s="32" t="n">
@@ -6319,12 +6376,12 @@
         <v>0.0136048066345096</v>
       </c>
       <c r="F49" s="30" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="23" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="B50" s="2"/>
       <c r="C50" s="24" t="n">
@@ -6340,12 +6397,12 @@
         <v>1782.85714285714</v>
       </c>
       <c r="F50" s="30" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="B52" s="8"/>
       <c r="C52" s="8"/>
@@ -6355,7 +6412,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
       <c r="B53" s="2"/>
       <c r="C53" s="22" t="n">
@@ -6374,7 +6431,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="23" t="s">
-        <v>398</v>
+        <v>403</v>
       </c>
       <c r="B54" s="2"/>
       <c r="C54" s="22" t="n">
@@ -6393,7 +6450,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="B55" s="2"/>
       <c r="C55" s="34" t="n">
@@ -6412,7 +6469,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="B56" s="2"/>
       <c r="C56" s="35" t="n">
@@ -6431,7 +6488,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23" t="s">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="B57" s="2"/>
       <c r="C57" s="35" t="n">
@@ -6450,7 +6507,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="23" t="s">
-        <v>402</v>
+        <v>407</v>
       </c>
       <c r="B58" s="2"/>
       <c r="C58" s="35" t="n">
@@ -6469,7 +6526,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="23" t="s">
-        <v>403</v>
+        <v>408</v>
       </c>
       <c r="B59" s="2"/>
       <c r="C59" s="35" t="n">
@@ -6488,7 +6545,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>404</v>
+        <v>409</v>
       </c>
       <c r="B60" s="2"/>
       <c r="C60" s="34" t="n">
@@ -6507,7 +6564,7 @@
     </row>
     <row r="61" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>405</v>
+        <v>410</v>
       </c>
       <c r="B61" s="2"/>
       <c r="C61" s="34" t="n">
@@ -6523,12 +6580,12 @@
         <v>1.01672535769804</v>
       </c>
       <c r="F61" s="30" t="s">
-        <v>406</v>
+        <v>411</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="23" t="s">
-        <v>407</v>
+        <v>412</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="35" t="n">
@@ -6544,12 +6601,12 @@
         <v>1.49945613983708</v>
       </c>
       <c r="F62" s="30" t="s">
-        <v>408</v>
+        <v>413</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>409</v>
+        <v>414</v>
       </c>
       <c r="B64" s="8"/>
       <c r="C64" s="8"/>
@@ -6559,7 +6616,7 @@
     </row>
     <row r="65" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="36" t="s">
-        <v>410</v>
+        <v>415</v>
       </c>
       <c r="B65" s="36"/>
       <c r="C65" s="36"/>
@@ -6569,7 +6626,7 @@
     </row>
     <row r="66" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="36" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="B66" s="36"/>
       <c r="C66" s="36"/>
@@ -6579,7 +6636,7 @@
     </row>
     <row r="67" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="36" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="B67" s="36"/>
       <c r="C67" s="36"/>
@@ -6589,7 +6646,7 @@
     </row>
     <row r="68" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="36" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="B68" s="36"/>
       <c r="C68" s="36"/>
@@ -6599,7 +6656,7 @@
     </row>
     <row r="69" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="36" t="s">
-        <v>414</v>
+        <v>419</v>
       </c>
       <c r="B69" s="36"/>
       <c r="C69" s="36"/>
@@ -6609,7 +6666,7 @@
     </row>
     <row r="70" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="36" t="s">
-        <v>415</v>
+        <v>420</v>
       </c>
       <c r="B70" s="36"/>
       <c r="C70" s="36"/>
@@ -6652,20 +6709,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>416</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>417</v>
+        <v>422</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>24</v>
@@ -6677,12 +6734,12 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>418</v>
+        <v>423</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -6692,7 +6749,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>419</v>
+        <v>424</v>
       </c>
       <c r="C6" s="24" t="n">
         <f aca="false">(Assumptions!$C$38*Assumptions!$C$44+Assumptions!$C$39*Assumptions!$C$45+Assumptions!$C$40*Assumptions!$C$46+Assumptions!$C$41*Assumptions!$C$47)/Assumptions!$C$42</f>
@@ -6710,7 +6767,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="C7" s="24" t="n">
         <f aca="false">Assumptions!$C$38+Assumptions!$C$39+Assumptions!$C$40+Assumptions!$C$41</f>
@@ -6725,12 +6782,12 @@
         <v>12376</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>421</v>
+        <v>426</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="C8" s="10" t="n">
         <f aca="false">0</f>
@@ -6748,7 +6805,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="C9" s="31" t="n">
         <f aca="false">C6/C7</f>
@@ -6763,12 +6820,12 @@
         <v>1.29464235422864</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>423</v>
+        <v>428</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>424</v>
+        <v>429</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -6778,7 +6835,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>425</v>
+        <v>430</v>
       </c>
       <c r="C12" s="24" t="n">
         <f aca="false">Tricity_Recon!C46</f>
@@ -6796,7 +6853,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>426</v>
+        <v>431</v>
       </c>
       <c r="C13" s="31" t="n">
         <f aca="false">Tricity_Recon!C47</f>
@@ -6814,7 +6871,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>427</v>
+        <v>432</v>
       </c>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -6824,7 +6881,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="23" t="s">
-        <v>428</v>
+        <v>433</v>
       </c>
       <c r="C16" s="24" t="n">
         <f aca="false">TAM_India!C31*Assumptions!$C$34/Assumptions!$C$33*Assumptions!$C$54</f>
@@ -6839,12 +6896,12 @@
         <v>10141.9872254916</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>429</v>
+        <v>434</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>430</v>
+        <v>435</v>
       </c>
       <c r="C17" s="25" t="n">
         <f aca="false">Assumptions!$C$68</f>
@@ -6862,7 +6919,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="s">
-        <v>431</v>
+        <v>436</v>
       </c>
       <c r="C18" s="24" t="n">
         <f aca="false">C16*C17</f>
@@ -6880,7 +6937,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="s">
-        <v>432</v>
+        <v>437</v>
       </c>
       <c r="C19" s="24" t="n">
         <f aca="false">Tricity_Recon!C48</f>
@@ -6895,12 +6952,12 @@
         <v>263.76</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>433</v>
+        <v>438</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>434</v>
+        <v>439</v>
       </c>
       <c r="C20" s="24" t="n">
         <f aca="false">MAX(0,C18-C19)</f>
@@ -6918,7 +6975,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="C21" s="31" t="n">
         <f aca="false">C20*Assumptions!$C$56/10000000</f>
@@ -6933,12 +6990,12 @@
         <v>10.5878246705899</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>436</v>
+        <v>441</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>437</v>
+        <v>442</v>
       </c>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -6948,7 +7005,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>438</v>
+        <v>443</v>
       </c>
       <c r="C24" s="24" t="n">
         <f aca="false">C16-C18</f>
@@ -6966,7 +7023,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>439</v>
+        <v>444</v>
       </c>
       <c r="C25" s="25" t="n">
         <f aca="false">Assumptions!$C$69</f>
@@ -6984,7 +7041,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="23" t="s">
-        <v>440</v>
+        <v>445</v>
       </c>
       <c r="C26" s="24" t="n">
         <f aca="false">C24*C25</f>
@@ -7002,7 +7059,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>441</v>
+        <v>446</v>
       </c>
       <c r="C27" s="31" t="n">
         <f aca="false">C26*Assumptions!$C$70/10000000</f>
@@ -7017,12 +7074,12 @@
         <v>5.84178464188316</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>442</v>
+        <v>447</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>443</v>
+        <v>448</v>
       </c>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -7032,7 +7089,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>444</v>
+        <v>449</v>
       </c>
       <c r="C30" s="24" t="n">
         <f aca="false">Assumptions!$C$71+Assumptions!$C$72</f>
@@ -7047,12 +7104,12 @@
         <v>5300</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>445</v>
+        <v>450</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>446</v>
+        <v>451</v>
       </c>
       <c r="C31" s="24" t="n">
         <f aca="false">C30*Assumptions!$C$73</f>
@@ -7070,7 +7127,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>447</v>
+        <v>452</v>
       </c>
       <c r="C32" s="31" t="n">
         <f aca="false">C31*Assumptions!$C$74/10000000</f>
@@ -7085,12 +7142,12 @@
         <v>2.544</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>448</v>
+        <v>453</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>449</v>
+        <v>454</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -7100,7 +7157,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>450</v>
+        <v>455</v>
       </c>
       <c r="C35" s="31" t="n">
         <f aca="false">TAM_India!C33*Assumptions!$C$75</f>
@@ -7115,12 +7172,12 @@
         <v>54</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>451</v>
+        <v>456</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="B37" s="8"/>
       <c r="C37" s="8"/>
@@ -7130,7 +7187,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="C38" s="31" t="n">
         <f aca="false">C13+C21+C27+C32</f>
@@ -7145,12 +7202,12 @@
         <v>24.2488093124731</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="23" t="s">
-        <v>455</v>
+        <v>460</v>
       </c>
       <c r="C39" s="22" t="n">
         <f aca="false">C35</f>
@@ -7165,12 +7222,12 @@
         <v>54</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>456</v>
+        <v>461</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>457</v>
+        <v>462</v>
       </c>
       <c r="C40" s="31" t="n">
         <f aca="false">C38+C39</f>
@@ -7188,7 +7245,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="23" t="s">
-        <v>458</v>
+        <v>463</v>
       </c>
       <c r="C41" s="24" t="n">
         <f aca="false">C12+C20+C26</f>
@@ -7206,7 +7263,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="23" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="C42" s="25" t="n">
         <f aca="false">C40/TAM_India!C34</f>
@@ -7224,7 +7281,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="23" t="s">
-        <v>460</v>
+        <v>465</v>
       </c>
       <c r="C43" s="22" t="n">
         <f aca="false">C13+C16*Assumptions!$C$56/10000000</f>
@@ -7239,12 +7296,12 @@
         <v>66.1271233529496</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>461</v>
+        <v>466</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="23" t="s">
-        <v>462</v>
+        <v>467</v>
       </c>
       <c r="C44" s="22" t="n">
         <f aca="false">TAM_India!C38*Assumptions!$C$56/TAM_India!C13</f>
@@ -7259,7 +7316,7 @@
         <v>57.834</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>463</v>
+        <v>468</v>
       </c>
     </row>
   </sheetData>
@@ -7278,7 +7335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -7289,37 +7346,37 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>464</v>
+        <v>469</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>465</v>
+        <v>470</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>466</v>
+        <v>471</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>467</v>
+        <v>472</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>468</v>
+        <v>473</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -7329,7 +7386,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="23" t="s">
-        <v>469</v>
+        <v>474</v>
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">Assumptions!$C$78*(1+Assumptions!$C$76)/100</f>
@@ -7344,12 +7401,12 @@
         <v>1.233926</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>470</v>
+        <v>475</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>471</v>
+        <v>476</v>
       </c>
       <c r="C7" s="37" t="n">
         <f aca="false">IFERROR(C6/SAM_North!C13,0)</f>
@@ -7367,7 +7424,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>472</v>
+        <v>477</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">Assumptions!$C$79*(1+Assumptions!$C$76)/100</f>
@@ -7382,12 +7439,12 @@
         <v>0.891608</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>473</v>
+        <v>478</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>474</v>
+        <v>479</v>
       </c>
       <c r="C9" s="37" t="n">
         <f aca="false">IFERROR(C8/SAM_North!C21,0)</f>
@@ -7405,7 +7462,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>475</v>
+        <v>480</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">Assumptions!$C$80*(1+Assumptions!$C$76)/100</f>
@@ -7420,12 +7477,12 @@
         <v>0.58233</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>476</v>
+        <v>481</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>477</v>
+        <v>482</v>
       </c>
       <c r="C11" s="37" t="n">
         <f aca="false">IFERROR(C10/SAM_North!C27,0)</f>
@@ -7443,7 +7500,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">Assumptions!$C$81*(1+Assumptions!$C$76)/100</f>
@@ -7458,12 +7515,12 @@
         <v>0.72157</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>479</v>
+        <v>484</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>480</v>
+        <v>485</v>
       </c>
       <c r="C13" s="37" t="n">
         <f aca="false">IFERROR(C12/SAM_North!C32,0)</f>
@@ -7481,7 +7538,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>481</v>
+        <v>486</v>
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">Assumptions!$C$82*(1+Assumptions!$C$76)/100</f>
@@ -7496,12 +7553,12 @@
         <v>0.399784</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>482</v>
+        <v>487</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>483</v>
+        <v>488</v>
       </c>
       <c r="C15" s="37" t="n">
         <f aca="false">IFERROR(C14/SAM_North!C35,0)</f>
@@ -7519,7 +7576,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>484</v>
+        <v>489</v>
       </c>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -7529,7 +7586,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>485</v>
+        <v>490</v>
       </c>
       <c r="C17" s="37" t="n">
         <f aca="false">Assumptions!$C$84/SAM_North!C12</f>
@@ -7544,12 +7601,12 @@
         <v>0.11089626933576</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>486</v>
+        <v>491</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>487</v>
+        <v>492</v>
       </c>
       <c r="C18" s="37" t="n">
         <f aca="false">IFERROR(Assumptions!$C$85/(SAM_North!C20+Tricity_Recon!C48),0)</f>
@@ -7564,12 +7621,12 @@
         <v>0.0468350027897985</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>488</v>
+        <v>493</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>489</v>
+        <v>494</v>
       </c>
       <c r="C19" s="37" t="n">
         <f aca="false">IFERROR(Assumptions!$C$86/SAM_North!C26,0)</f>
@@ -7587,7 +7644,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="C20" s="25" t="n">
         <f aca="false">Assumptions!$C$84/Tricity_Recon!C15</f>
@@ -7605,7 +7662,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="C21" s="31" t="n">
         <f aca="false">C6+C8+C10+C12+C14</f>
@@ -7623,7 +7680,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="C22" s="37" t="n">
         <f aca="false">(C21-C14)/SAM_North!C38</f>
@@ -7641,7 +7698,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>493</v>
+        <v>498</v>
       </c>
       <c r="C23" s="25" t="n">
         <f aca="false">C21/SAM_North!C40</f>
@@ -7659,7 +7716,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="23" t="s">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="C24" s="33" t="n">
         <f aca="false">C21/TAM_India!C34</f>
@@ -7674,12 +7731,12 @@
         <v>0.0025640940136601</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>495</v>
+        <v>500</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="23" t="s">
-        <v>496</v>
+        <v>501</v>
       </c>
       <c r="C25" s="22" t="n">
         <f aca="false">Assumptions!$C$83*(1+Assumptions!$C$76)/100</f>
@@ -7694,12 +7751,12 @@
         <v>0.119534</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>497</v>
+        <v>502</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>498</v>
+        <v>503</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -7709,27 +7766,27 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="23" t="s">
-        <v>499</v>
+        <v>504</v>
       </c>
       <c r="C28" s="22" t="n">
-        <f aca="false">Assumptions!$C$87*(1+Assumptions!$C$76)/100</f>
+        <f aca="false">Assumptions!$C$88*(1+Assumptions!$C$76)/100</f>
         <v>0.079178</v>
       </c>
       <c r="D28" s="22" t="n">
-        <f aca="false">Assumptions!$D$87*(1+Assumptions!$D$76)/100</f>
+        <f aca="false">Assumptions!$D$88*(1+Assumptions!$D$76)/100</f>
         <v>0.195998</v>
       </c>
       <c r="E28" s="22" t="n">
-        <f aca="false">Assumptions!$E$87*(1+Assumptions!$E$76)/100</f>
+        <f aca="false">Assumptions!$E$88*(1+Assumptions!$E$76)/100</f>
         <v>0.294056</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>500</v>
+        <v>505</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>501</v>
+        <v>506</v>
       </c>
       <c r="C29" s="37" t="n">
         <f aca="false">C28/SAM_North!C13</f>
@@ -7744,12 +7801,12 @@
         <v>0.0557430997876858</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>502</v>
+        <v>507</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="23" t="s">
-        <v>503</v>
+        <v>508</v>
       </c>
       <c r="C30" s="35" t="n">
         <f aca="false">IFERROR(C21/C28,0)</f>
@@ -7765,9 +7822,29 @@
       </c>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>504</v>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>509</v>
+      </c>
+      <c r="C31" s="37" t="n">
+        <f aca="false">Assumptions!$C$87/Tricity_Recon!$E$46</f>
+        <v>0.0341219290263876</v>
+      </c>
+      <c r="D31" s="37" t="n">
+        <f aca="false">Assumptions!$D$87/Tricity_Recon!$D$46</f>
+        <v>0.0688593214696274</v>
+      </c>
+      <c r="E31" s="37" t="n">
+        <f aca="false">Assumptions!$E$87/Tricity_Recon!$C$46</f>
+        <v>0.123901838835178</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="2" t="s">
+        <v>511</v>
       </c>
     </row>
   </sheetData>
@@ -7786,7 +7863,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
@@ -7798,17 +7875,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6" t="s">
@@ -7821,15 +7898,15 @@
         <v>25</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="C5" s="29" t="n">
         <f aca="false">TAM_India!C30</f>
@@ -7848,12 +7925,12 @@
         <v>387.7453125</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="C6" s="29" t="n">
         <f aca="false">TAM_India!C33</f>
@@ -7872,12 +7949,12 @@
         <v>22.5</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="C7" s="29" t="n">
         <f aca="false">TAM_India!C38</f>
@@ -7896,12 +7973,12 @@
         <v>29.66251640625</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">SAM_North!C40</f>
@@ -7920,12 +7997,12 @@
         <v>15.6698825661453</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="C9" s="22" t="n">
         <f aca="false">SAM_North!C38</f>
@@ -7944,12 +8021,12 @@
         <v>7.79488256614533</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">SAM_North!C13</f>
@@ -7968,12 +8045,12 @@
         <v>3.26753147138174</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="C11" s="22" t="n">
         <f aca="false">SAM_North!C21</f>
@@ -7992,12 +8069,12 @@
         <v>1.93913479201771</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">SAM_North!C27</f>
@@ -8019,7 +8096,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="C13" s="22" t="n">
         <f aca="false">SAM_North!C32</f>
@@ -8038,12 +8115,12 @@
         <v>1.2</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">SAM_North!C35</f>
@@ -8065,7 +8142,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="C15" s="22" t="n">
         <f aca="false">SOM_PNA!C21</f>
@@ -8084,12 +8161,12 @@
         <v>1.892484</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="C16" s="25" t="n">
         <f aca="false">SOM_PNA!C22</f>
@@ -8111,7 +8188,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="C17" s="25" t="n">
         <f aca="false">SOM_PNA!C17</f>
@@ -8130,12 +8207,12 @@
         <v>0.12931780571996</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="C18" s="33" t="n">
         <f aca="false">SOM_PNA!C24</f>
@@ -8157,7 +8234,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="C19" s="22" t="n">
         <f aca="false">SOM_PNA!C28</f>
@@ -8176,56 +8253,80 @@
         <v>0.195998</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>535</v>
-      </c>
-      <c r="C20" s="24" t="n">
+      <c r="A20" s="0" t="s">
+        <v>542</v>
+      </c>
+      <c r="C20" s="25" t="n">
+        <f aca="false">SOM_PNA!C31</f>
+        <v>0.0341219290263876</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <f aca="false">SOM_PNA!D31</f>
+        <v>0.0688593214696274</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <f aca="false">SOM_PNA!E31</f>
+        <v>0.123901838835178</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <f aca="false">INDEX(C20:E20,Assumptions!$C$4)</f>
+        <v>0.0688593214696274</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
+        <v>544</v>
+      </c>
+      <c r="C21" s="24" t="n">
         <f aca="false">TAM_India!C31</f>
         <v>20100</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D21" s="24" t="n">
         <f aca="false">TAM_India!D31</f>
         <v>56812.5</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E21" s="24" t="n">
         <f aca="false">TAM_India!E31</f>
         <v>126000</v>
       </c>
-      <c r="F20" s="11" t="n">
-        <f aca="false">INDEX(C20:E20,Assumptions!$C$4)</f>
+      <c r="F21" s="11" t="n">
+        <f aca="false">INDEX(C21:E21,Assumptions!$C$4)</f>
         <v>56812.5</v>
       </c>
-      <c r="G20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="C21" s="24" t="n">
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>545</v>
+      </c>
+      <c r="C22" s="24" t="n">
         <f aca="false">Tricity_Recon!C46</f>
         <v>484.254314254494</v>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D22" s="24" t="n">
         <f aca="false">Tricity_Recon!D46</f>
         <v>726.118104751498</v>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E22" s="24" t="n">
         <f aca="false">Tricity_Recon!E46</f>
         <v>879.2</v>
       </c>
-      <c r="F21" s="11" t="n">
-        <f aca="false">INDEX(C21:E21,Assumptions!$C$4)</f>
+      <c r="F22" s="11" t="n">
+        <f aca="false">INDEX(C22:E22,Assumptions!$C$4)</f>
         <v>726.118104751498</v>
       </c>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>537</v>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="2" t="s">
+        <v>546</v>
       </c>
     </row>
   </sheetData>
@@ -8256,29 +8357,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>538</v>
+        <v>547</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>539</v>
+        <v>548</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>540</v>
+        <v>549</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>541</v>
+        <v>550</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>542</v>
+        <v>551</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>543</v>
+        <v>552</v>
       </c>
       <c r="B5" s="29" t="n">
         <v>276999</v>
@@ -8287,15 +8388,15 @@
         <v>105</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>545</v>
+        <v>554</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
       <c r="B6" s="29" t="n">
         <v>76141</v>
@@ -8304,49 +8405,49 @@
         <v>105</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>547</v>
+        <v>556</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="B7" s="29" t="n">
         <v>1.52</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>550</v>
+        <v>559</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>551</v>
+        <v>560</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>552</v>
+        <v>561</v>
       </c>
       <c r="B8" s="29" t="n">
         <v>12.6</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>553</v>
+        <v>562</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>555</v>
+        <v>564</v>
       </c>
       <c r="B9" s="29" t="n">
         <v>2880</v>
@@ -8355,15 +8456,15 @@
         <v>105</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>556</v>
+        <v>565</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>557</v>
+        <v>566</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>558</v>
+        <v>567</v>
       </c>
       <c r="B10" s="29" t="n">
         <v>650000</v>
@@ -8372,15 +8473,15 @@
         <v>105</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>559</v>
+        <v>568</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>560</v>
+        <v>569</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>561</v>
+        <v>570</v>
       </c>
       <c r="B11" s="29" t="n">
         <f aca="false">TAM_India!D36</f>
@@ -8390,15 +8491,15 @@
         <v>105</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>562</v>
+        <v>571</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>563</v>
+        <v>572</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>564</v>
+        <v>573</v>
       </c>
       <c r="B13" s="29" t="n">
         <f aca="false">TAM_India!D30</f>
@@ -8431,23 +8532,23 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>565</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>566</v>
+        <v>575</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>567</v>
+        <v>576</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>568</v>
+        <v>577</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>569</v>
+        <v>578</v>
       </c>
       <c r="B5" s="38" t="b">
         <f aca="false">ABS(TAM_India!D14-522.1)&lt;1</f>
@@ -8456,7 +8557,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>570</v>
+        <v>579</v>
       </c>
       <c r="B6" s="38" t="b">
         <f aca="false">ABS(TAM_India!D30-387.7)&lt;1</f>
@@ -8465,7 +8566,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>571</v>
+        <v>580</v>
       </c>
       <c r="B7" s="38" t="b">
         <f aca="false">ABS(Tricity_Recon!D16-5.65)&lt;0.1</f>
@@ -8474,7 +8575,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="B8" s="38" t="b">
         <f aca="false">AND(Tricity_Recon!D46&gt;=Tricity_Recon!D28,Tricity_Recon!D46&lt;=Tricity_Recon!D34)</f>
@@ -8483,7 +8584,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>573</v>
+        <v>582</v>
       </c>
       <c r="B9" s="38" t="b">
         <f aca="false">AND(Tricity_Recon!C47&lt;=Tricity_Recon!D47,Tricity_Recon!D47&lt;=Tricity_Recon!E47)</f>
@@ -8492,7 +8593,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="B10" s="38" t="b">
         <f aca="false">AND(SAM_North!C40&lt;TAM_India!C34,SAM_North!D40&lt;TAM_India!D34,SAM_North!E40&lt;TAM_India!E34)</f>
@@ -8501,7 +8602,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>575</v>
+        <v>584</v>
       </c>
       <c r="B11" s="38" t="b">
         <f aca="false">AND(SOM_PNA!C21&lt;SAM_North!C40,SOM_PNA!D21&lt;SAM_North!D40,SOM_PNA!E21&lt;SAM_North!E40)</f>
@@ -8510,7 +8611,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>576</v>
+        <v>585</v>
       </c>
       <c r="B12" s="38" t="b">
         <f aca="false">SOM_PNA!D17&lt;=0.25</f>
@@ -8519,7 +8620,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>577</v>
+        <v>586</v>
       </c>
       <c r="B13" s="38" t="b">
         <f aca="false">ABS(Tricity_Recon!D12/Tricity_Recon!D10-1)&lt;0.1</f>
@@ -8528,7 +8629,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>578</v>
+        <v>587</v>
       </c>
       <c r="B15" s="38" t="b">
         <f aca="false">AND(B5:B13)</f>

</xml_diff>

<commit_message>
Add Staged Plan economics run and align media spend to channel plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K2weV5RtvDCshBNnABKa1E
</commit_message>
<xml_diff>
--- a/priyanka_nanda_academy/economics/market_sizing_model.xlsx
+++ b/priyanka_nanda_academy/economics/market_sizing_model.xlsx
@@ -4582,7 +4582,7 @@
         <v>19.51</v>
       </c>
       <c r="D78" s="16" t="n">
-        <v>71.88</v>
+        <v>70.9</v>
       </c>
       <c r="E78" s="16" t="n">
         <v>104.57</v>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="I78" s="17" t="n">
         <f aca="false">INDEX(C78:E78,$C$4)</f>
-        <v>71.88</v>
+        <v>70.9</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4612,7 +4612,7 @@
         <v>3.4</v>
       </c>
       <c r="D79" s="16" t="n">
-        <v>24.86</v>
+        <v>24.45</v>
       </c>
       <c r="E79" s="16" t="n">
         <v>75.56</v>
@@ -4628,7 +4628,7 @@
       </c>
       <c r="I79" s="17" t="n">
         <f aca="false">INDEX(C79:E79,$C$4)</f>
-        <v>24.86</v>
+        <v>24.45</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4672,7 +4672,7 @@
         <v>5.84</v>
       </c>
       <c r="D81" s="16" t="n">
-        <v>27.06</v>
+        <v>27.04</v>
       </c>
       <c r="E81" s="16" t="n">
         <v>61.15</v>
@@ -4688,7 +4688,7 @@
       </c>
       <c r="I81" s="17" t="n">
         <f aca="false">INDEX(C81:E81,$C$4)</f>
-        <v>27.06</v>
+        <v>27.04</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4732,7 +4732,7 @@
         <v>2</v>
       </c>
       <c r="D83" s="16" t="n">
-        <v>6.55</v>
+        <v>6.54</v>
       </c>
       <c r="E83" s="16" t="n">
         <v>10.13</v>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="I83" s="17" t="n">
         <f aca="false">INDEX(C83:E83,$C$4)</f>
-        <v>6.55</v>
+        <v>6.54</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4762,7 +4762,7 @@
         <v>33.6</v>
       </c>
       <c r="D84" s="9" t="n">
-        <v>93.9</v>
+        <v>92.3</v>
       </c>
       <c r="E84" s="9" t="n">
         <v>97.5</v>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="I84" s="11" t="n">
         <f aca="false">INDEX(C84:E84,$C$4)</f>
-        <v>93.9</v>
+        <v>92.3</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4792,7 +4792,7 @@
         <v>7.4</v>
       </c>
       <c r="D85" s="9" t="n">
-        <v>40.2</v>
+        <v>39.6</v>
       </c>
       <c r="E85" s="9" t="n">
         <v>95</v>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="I85" s="11" t="n">
         <f aca="false">INDEX(C85:E85,$C$4)</f>
-        <v>40.2</v>
+        <v>39.6</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="D6" s="22" t="n">
         <f aca="false">Assumptions!$D$78*(1+Assumptions!$D$76)/100</f>
-        <v>0.848184</v>
+        <v>0.83662</v>
       </c>
       <c r="E6" s="22" t="n">
         <f aca="false">Assumptions!$E$78*(1+Assumptions!$E$76)/100</f>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="D7" s="37" t="n">
         <f aca="false">IFERROR(D6/SAM_North!D13,0)</f>
-        <v>0.259579443206198</v>
+        <v>0.256040380124088</v>
       </c>
       <c r="E7" s="37" t="n">
         <f aca="false">IFERROR(E6/SAM_North!E13,0)</f>
@@ -7432,7 +7432,7 @@
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">Assumptions!$D$79*(1+Assumptions!$D$76)/100</f>
-        <v>0.293348</v>
+        <v>0.28851</v>
       </c>
       <c r="E8" s="22" t="n">
         <f aca="false">Assumptions!$E$79*(1+Assumptions!$E$76)/100</f>
@@ -7452,7 +7452,7 @@
       </c>
       <c r="D9" s="37" t="n">
         <f aca="false">IFERROR(D8/SAM_North!D21,0)</f>
-        <v>0.151277776670061</v>
+        <v>0.148782849540748</v>
       </c>
       <c r="E9" s="37" t="n">
         <f aca="false">IFERROR(E8/SAM_North!E21,0)</f>
@@ -7508,7 +7508,7 @@
       </c>
       <c r="D12" s="22" t="n">
         <f aca="false">Assumptions!$D$81*(1+Assumptions!$D$76)/100</f>
-        <v>0.319308</v>
+        <v>0.319072</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">Assumptions!$E$81*(1+Assumptions!$E$76)/100</f>
@@ -7528,7 +7528,7 @@
       </c>
       <c r="D13" s="37" t="n">
         <f aca="false">IFERROR(D12/SAM_North!D32,0)</f>
-        <v>0.26609</v>
+        <v>0.265893333333333</v>
       </c>
       <c r="E13" s="37" t="n">
         <f aca="false">IFERROR(E12/SAM_North!E32,0)</f>
@@ -7594,7 +7594,7 @@
       </c>
       <c r="D17" s="37" t="n">
         <f aca="false">Assumptions!$D$84/SAM_North!D12</f>
-        <v>0.12931780571996</v>
+        <v>0.127114307432932</v>
       </c>
       <c r="E17" s="37" t="n">
         <f aca="false">Assumptions!$E$84/SAM_North!E12</f>
@@ -7614,7 +7614,7 @@
       </c>
       <c r="D18" s="37" t="n">
         <f aca="false">IFERROR(Assumptions!$D$85/(SAM_North!D20+Tricity_Recon!D48),0)</f>
-        <v>0.0656381860807753</v>
+        <v>0.0646585116616593</v>
       </c>
       <c r="E18" s="37" t="n">
         <f aca="false">IFERROR(Assumptions!$E$85/(SAM_North!E20+Tricity_Recon!E48),0)</f>
@@ -7652,7 +7652,7 @@
       </c>
       <c r="D20" s="25" t="n">
         <f aca="false">Assumptions!$D$84/Tricity_Recon!D15</f>
-        <v>0.0747611464968153</v>
+        <v>0.0734872611464968</v>
       </c>
       <c r="E20" s="25" t="n">
         <f aca="false">Assumptions!$E$84/Tricity_Recon!E15</f>
@@ -7670,7 +7670,7 @@
       </c>
       <c r="D21" s="31" t="n">
         <f aca="false">D6+D8+D10+D12+D14</f>
-        <v>1.892484</v>
+        <v>1.875846</v>
       </c>
       <c r="E21" s="31" t="n">
         <f aca="false">E6+E8+E10+E12+E14</f>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="D22" s="37" t="n">
         <f aca="false">(D21-D14)/SAM_North!D38</f>
-        <v>0.22548255026107</v>
+        <v>0.22334807294742</v>
       </c>
       <c r="E22" s="37" t="n">
         <f aca="false">(E21-E14)/SAM_North!E38</f>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="D23" s="25" t="n">
         <f aca="false">D21/SAM_North!D40</f>
-        <v>0.120772060161363</v>
+        <v>0.119710278113555</v>
       </c>
       <c r="E23" s="25" t="n">
         <f aca="false">E21/SAM_North!E40</f>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="D24" s="33" t="n">
         <f aca="false">D21/TAM_India!D34</f>
-        <v>0.00461305453672917</v>
+        <v>0.00457249831465168</v>
       </c>
       <c r="E24" s="33" t="n">
         <f aca="false">E21/TAM_India!E34</f>
@@ -7744,7 +7744,7 @@
       </c>
       <c r="D25" s="22" t="n">
         <f aca="false">Assumptions!$D$83*(1+Assumptions!$D$76)/100</f>
-        <v>0.07729</v>
+        <v>0.077172</v>
       </c>
       <c r="E25" s="22" t="n">
         <f aca="false">Assumptions!$E$83*(1+Assumptions!$E$76)/100</f>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="D30" s="35" t="n">
         <f aca="false">IFERROR(D21/D28,0)</f>
-        <v>9.65562913907285</v>
+        <v>9.57074051776039</v>
       </c>
       <c r="E30" s="35" t="n">
         <f aca="false">IFERROR(E21/E28,0)</f>
@@ -8150,7 +8150,7 @@
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">SOM_PNA!D21</f>
-        <v>1.892484</v>
+        <v>1.875846</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">SOM_PNA!E21</f>
@@ -8158,7 +8158,7 @@
       </c>
       <c r="F15" s="21" t="n">
         <f aca="false">INDEX(C15:E15,Assumptions!$C$4)</f>
-        <v>1.892484</v>
+        <v>1.875846</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>535</v>
@@ -8174,7 +8174,7 @@
       </c>
       <c r="D16" s="25" t="n">
         <f aca="false">SOM_PNA!D22</f>
-        <v>0.22548255026107</v>
+        <v>0.22334807294742</v>
       </c>
       <c r="E16" s="25" t="n">
         <f aca="false">SOM_PNA!E22</f>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="F16" s="13" t="n">
         <f aca="false">INDEX(C16:E16,Assumptions!$C$4)</f>
-        <v>0.22548255026107</v>
+        <v>0.22334807294742</v>
       </c>
       <c r="G16" s="2"/>
     </row>
@@ -8196,7 +8196,7 @@
       </c>
       <c r="D17" s="25" t="n">
         <f aca="false">SOM_PNA!D17</f>
-        <v>0.12931780571996</v>
+        <v>0.127114307432932</v>
       </c>
       <c r="E17" s="25" t="n">
         <f aca="false">SOM_PNA!E17</f>
@@ -8204,7 +8204,7 @@
       </c>
       <c r="F17" s="13" t="n">
         <f aca="false">INDEX(C17:E17,Assumptions!$C$4)</f>
-        <v>0.12931780571996</v>
+        <v>0.127114307432932</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>538</v>
@@ -8220,7 +8220,7 @@
       </c>
       <c r="D18" s="33" t="n">
         <f aca="false">SOM_PNA!D24</f>
-        <v>0.00461305453672917</v>
+        <v>0.00457249831465168</v>
       </c>
       <c r="E18" s="33" t="n">
         <f aca="false">SOM_PNA!E24</f>
@@ -8228,7 +8228,7 @@
       </c>
       <c r="F18" s="19" t="n">
         <f aca="false">INDEX(C18:E18,Assumptions!$C$4)</f>
-        <v>0.00461305453672917</v>
+        <v>0.00457249831465168</v>
       </c>
       <c r="G18" s="2"/>
     </row>

</xml_diff>